<commit_message>
Updated training loss landscape code
</commit_message>
<xml_diff>
--- a/documents/results_raw_two_seeds.xlsx
+++ b/documents/results_raw_two_seeds.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Nagc2/Desktop/so101-vla-data-study/documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED11B206-1E70-9D4E-BD24-30320E99DFC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA1062B2-B25B-4745-BC16-0A6CD7E9AE07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20" yWindow="700" windowWidth="17120" windowHeight="20180" activeTab="2" xr2:uid="{E9882473-D8D3-4249-9541-943B7997CA3D}"/>
+    <workbookView xWindow="16720" yWindow="720" windowWidth="17120" windowHeight="20180" activeTab="2" xr2:uid="{E9882473-D8D3-4249-9541-943B7997CA3D}"/>
   </bookViews>
   <sheets>
     <sheet name="results" sheetId="1" r:id="rId1"/>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6646" uniqueCount="386">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6625" uniqueCount="377">
   <si>
     <t>condition</t>
   </si>
@@ -562,9 +562,6 @@
     <t xml:space="preserve">believe it missed th cube entierely and went to the top </t>
   </si>
   <si>
-    <t>review</t>
-  </si>
-  <si>
     <t>took a few seconds to get back to prose position</t>
   </si>
   <si>
@@ -580,9 +577,6 @@
     <t>Dropp[ed cube next to cup, accidentally ended episode early</t>
   </si>
   <si>
-    <t>accidental key press, after failure happened</t>
-  </si>
-  <si>
     <t>missed cube and went to the top of board</t>
   </si>
   <si>
@@ -601,9 +595,6 @@
     <t xml:space="preserve">Bumped cube and went up towards middle </t>
   </si>
   <si>
-    <t>confirm didn't touch cube</t>
-  </si>
-  <si>
     <t>missed the cube went to top of board</t>
   </si>
   <si>
@@ -613,9 +604,6 @@
     <t>bumped cube, went to cup, then went back and got the cube, it fell on the edge and rolled int</t>
   </si>
   <si>
-    <t>check recording, rerecorded because of doube right click</t>
-  </si>
-  <si>
     <t>went towards t4 after bumping cube</t>
   </si>
   <si>
@@ -634,9 +622,6 @@
     <t>Bumped cube and went to T4 and center of table</t>
   </si>
   <si>
-    <t>confrim contact</t>
-  </si>
-  <si>
     <t>bumped cube, moved as if it went to the cup, then to T4 and cneter</t>
   </si>
   <si>
@@ -739,9 +724,6 @@
     <t>went between e5 and t7</t>
   </si>
   <si>
-    <t>cvonfirm</t>
-  </si>
-  <si>
     <t>Went to T2 then rotated to T1</t>
   </si>
   <si>
@@ -820,9 +802,6 @@
     <t>missed the cube slightly</t>
   </si>
   <si>
-    <t>confirm if it bumped cube or not</t>
-  </si>
-  <si>
     <t xml:space="preserve">bumped cube, missed </t>
   </si>
   <si>
@@ -841,9 +820,6 @@
     <t>bumped cube and missed, ended at T4</t>
   </si>
   <si>
-    <t>confirm no contact</t>
-  </si>
-  <si>
     <t>went to cube but passed over it</t>
   </si>
   <si>
@@ -865,9 +841,6 @@
     <t>aimed to the left</t>
   </si>
   <si>
-    <t>confirm contact</t>
-  </si>
-  <si>
     <t>likely aimed at cube, ended at T3, to confirm intiial motion and contact</t>
   </si>
   <si>
@@ -928,9 +901,6 @@
     <t>took a second to depart</t>
   </si>
   <si>
-    <t>confirm</t>
-  </si>
-  <si>
     <t>went too high and missed the cube</t>
   </si>
   <si>
@@ -1063,9 +1033,6 @@
     <t>went to t10, then to cube but not far enough</t>
   </si>
   <si>
-    <t>error happened, following ones were appended</t>
-  </si>
-  <si>
     <t>aimed between t7 and e5, then t7</t>
   </si>
   <si>
@@ -1129,9 +1096,6 @@
     <t>went to t2, bumped cup, went to prose</t>
   </si>
   <si>
-    <t>cup may have been shifted a bit, didn't seem to affect performance based on other videos</t>
-  </si>
-  <si>
     <t>aimed to the right of cube before going up to T3</t>
   </si>
   <si>
@@ -1226,6 +1190,15 @@
   </si>
   <si>
     <t>went closer to t7, then to t4</t>
+  </si>
+  <si>
+    <t>aimed left, seems to have hit cube, difficult to see on video</t>
+  </si>
+  <si>
+    <t>went middle, seems to have pushed the cube slightly downward</t>
+  </si>
+  <si>
+    <t>went to t1, cup started 1 inch higher than the position it should be in</t>
   </si>
 </sst>
 </file>
@@ -21156,9 +21129,6 @@
       <c r="F19">
         <v>0</v>
       </c>
-      <c r="G19" t="s">
-        <v>164</v>
-      </c>
       <c r="H19" t="s">
         <v>62</v>
       </c>
@@ -21212,7 +21182,7 @@
         <v>13</v>
       </c>
       <c r="J21" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.2">
@@ -21261,7 +21231,7 @@
         <v>62</v>
       </c>
       <c r="J23" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.2">
@@ -21287,7 +21257,7 @@
         <v>59</v>
       </c>
       <c r="J24" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.2">
@@ -21313,7 +21283,7 @@
         <v>62</v>
       </c>
       <c r="J25" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.2">
@@ -21358,14 +21328,11 @@
       <c r="F27">
         <v>0</v>
       </c>
-      <c r="G27" t="s">
-        <v>170</v>
-      </c>
       <c r="H27" t="s">
         <v>59</v>
       </c>
       <c r="J27" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.2">
@@ -21460,7 +21427,7 @@
         <v>62</v>
       </c>
       <c r="J31" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.2">
@@ -21578,7 +21545,7 @@
         <v>58</v>
       </c>
       <c r="J36" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.2">
@@ -21604,7 +21571,7 @@
         <v>58</v>
       </c>
       <c r="J37" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.2">
@@ -21630,7 +21597,7 @@
         <v>62</v>
       </c>
       <c r="J38" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.2">
@@ -21656,7 +21623,7 @@
         <v>62</v>
       </c>
       <c r="J39" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.2">
@@ -21682,7 +21649,7 @@
         <v>62</v>
       </c>
       <c r="J40" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.2">
@@ -21708,7 +21675,7 @@
         <v>62</v>
       </c>
       <c r="J41" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.2">
@@ -21734,7 +21701,7 @@
         <v>62</v>
       </c>
       <c r="J42" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.2">
@@ -21760,7 +21727,7 @@
         <v>62</v>
       </c>
       <c r="J43" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.2">
@@ -21786,7 +21753,7 @@
         <v>62</v>
       </c>
       <c r="J44" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.2">
@@ -21812,7 +21779,7 @@
         <v>62</v>
       </c>
       <c r="J45" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.2">
@@ -21838,7 +21805,7 @@
         <v>62</v>
       </c>
       <c r="J46" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.2">
@@ -21864,7 +21831,7 @@
         <v>62</v>
       </c>
       <c r="J47" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.2">
@@ -21890,7 +21857,7 @@
         <v>62</v>
       </c>
       <c r="J48" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.2">
@@ -21916,7 +21883,7 @@
         <v>62</v>
       </c>
       <c r="J49" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.2">
@@ -21942,7 +21909,7 @@
         <v>62</v>
       </c>
       <c r="J50" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.2">
@@ -21968,7 +21935,7 @@
         <v>62</v>
       </c>
       <c r="J51" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.2">
@@ -21994,7 +21961,7 @@
         <v>62</v>
       </c>
       <c r="J52" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.2">
@@ -22020,7 +21987,7 @@
         <v>62</v>
       </c>
       <c r="J53" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.2">
@@ -22046,7 +22013,7 @@
         <v>62</v>
       </c>
       <c r="J54" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.2">
@@ -22072,7 +22039,7 @@
         <v>62</v>
       </c>
       <c r="J55" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.2">
@@ -22098,7 +22065,7 @@
         <v>62</v>
       </c>
       <c r="J56" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.2">
@@ -22124,7 +22091,7 @@
         <v>62</v>
       </c>
       <c r="J57" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.2">
@@ -22176,7 +22143,7 @@
         <v>62</v>
       </c>
       <c r="J59" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.2">
@@ -22634,7 +22601,7 @@
         <v>58</v>
       </c>
       <c r="J78" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="79" spans="1:12" x14ac:dyDescent="0.2">
@@ -22660,7 +22627,7 @@
         <v>13</v>
       </c>
       <c r="L79" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
     </row>
     <row r="80" spans="1:12" x14ac:dyDescent="0.2">
@@ -22732,7 +22699,7 @@
         <v>58</v>
       </c>
       <c r="J82" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="83" spans="1:10" x14ac:dyDescent="0.2">
@@ -22758,7 +22725,7 @@
         <v>13</v>
       </c>
       <c r="J83" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
     </row>
     <row r="84" spans="1:10" x14ac:dyDescent="0.2">
@@ -22784,7 +22751,7 @@
         <v>58</v>
       </c>
       <c r="J84" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
     </row>
     <row r="85" spans="1:10" x14ac:dyDescent="0.2">
@@ -22829,14 +22796,11 @@
       <c r="F86">
         <v>0</v>
       </c>
-      <c r="G86" t="s">
-        <v>177</v>
-      </c>
       <c r="H86" t="s">
         <v>62</v>
       </c>
       <c r="J86" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="87" spans="1:10" x14ac:dyDescent="0.2">
@@ -22862,7 +22826,7 @@
         <v>13</v>
       </c>
       <c r="J87" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
     </row>
     <row r="88" spans="1:10" x14ac:dyDescent="0.2">
@@ -22888,7 +22852,7 @@
         <v>56</v>
       </c>
       <c r="J88" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
     </row>
     <row r="89" spans="1:10" x14ac:dyDescent="0.2">
@@ -22933,14 +22897,11 @@
       <c r="F90">
         <v>0</v>
       </c>
-      <c r="G90" t="s">
-        <v>181</v>
-      </c>
       <c r="H90" t="s">
         <v>58</v>
       </c>
       <c r="J90" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
     </row>
     <row r="91" spans="1:10" x14ac:dyDescent="0.2">
@@ -22989,7 +22950,7 @@
         <v>58</v>
       </c>
       <c r="J92" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
     </row>
     <row r="93" spans="1:10" x14ac:dyDescent="0.2">
@@ -23153,7 +23114,7 @@
         <v>62</v>
       </c>
       <c r="J99" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
     </row>
     <row r="100" spans="1:10" x14ac:dyDescent="0.2">
@@ -23179,7 +23140,7 @@
         <v>62</v>
       </c>
       <c r="J100" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
     </row>
     <row r="101" spans="1:10" x14ac:dyDescent="0.2">
@@ -23205,7 +23166,7 @@
         <v>62</v>
       </c>
       <c r="J101" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
     </row>
     <row r="102" spans="1:10" x14ac:dyDescent="0.2">
@@ -23231,7 +23192,7 @@
         <v>58</v>
       </c>
       <c r="J102" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
     </row>
     <row r="103" spans="1:10" x14ac:dyDescent="0.2">
@@ -23257,7 +23218,7 @@
         <v>62</v>
       </c>
       <c r="J103" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
     </row>
     <row r="104" spans="1:10" x14ac:dyDescent="0.2">
@@ -23283,7 +23244,7 @@
         <v>62</v>
       </c>
       <c r="J104" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
     </row>
     <row r="105" spans="1:10" x14ac:dyDescent="0.2">
@@ -23309,7 +23270,7 @@
         <v>62</v>
       </c>
       <c r="J105" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
     </row>
     <row r="106" spans="1:10" x14ac:dyDescent="0.2">
@@ -23335,7 +23296,7 @@
         <v>62</v>
       </c>
       <c r="J106" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
     </row>
     <row r="107" spans="1:10" x14ac:dyDescent="0.2">
@@ -23361,7 +23322,7 @@
         <v>62</v>
       </c>
       <c r="J107" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
     </row>
     <row r="108" spans="1:10" x14ac:dyDescent="0.2">
@@ -23387,7 +23348,7 @@
         <v>62</v>
       </c>
       <c r="J108" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
     </row>
     <row r="109" spans="1:10" x14ac:dyDescent="0.2">
@@ -23413,7 +23374,7 @@
         <v>62</v>
       </c>
       <c r="J109" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
     </row>
     <row r="110" spans="1:10" x14ac:dyDescent="0.2">
@@ -23439,7 +23400,7 @@
         <v>62</v>
       </c>
       <c r="J110" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
     </row>
     <row r="111" spans="1:10" x14ac:dyDescent="0.2">
@@ -23465,7 +23426,7 @@
         <v>62</v>
       </c>
       <c r="J111" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
     </row>
     <row r="112" spans="1:10" x14ac:dyDescent="0.2">
@@ -23491,7 +23452,7 @@
         <v>58</v>
       </c>
       <c r="J112" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
     </row>
     <row r="113" spans="1:10" x14ac:dyDescent="0.2">
@@ -23517,7 +23478,7 @@
         <v>62</v>
       </c>
       <c r="J113" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
     </row>
     <row r="114" spans="1:10" x14ac:dyDescent="0.2">
@@ -23543,7 +23504,7 @@
         <v>62</v>
       </c>
       <c r="J114" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
     </row>
     <row r="115" spans="1:10" x14ac:dyDescent="0.2">
@@ -23569,7 +23530,7 @@
         <v>62</v>
       </c>
       <c r="J115" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
     </row>
     <row r="116" spans="1:10" x14ac:dyDescent="0.2">
@@ -23595,7 +23556,7 @@
         <v>62</v>
       </c>
       <c r="J116" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
     </row>
     <row r="117" spans="1:10" x14ac:dyDescent="0.2">
@@ -23621,7 +23582,7 @@
         <v>62</v>
       </c>
       <c r="J117" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
     </row>
     <row r="118" spans="1:10" x14ac:dyDescent="0.2">
@@ -23643,14 +23604,11 @@
       <c r="F118">
         <v>0</v>
       </c>
-      <c r="G118" t="s">
-        <v>223</v>
-      </c>
       <c r="H118" t="s">
         <v>62</v>
       </c>
       <c r="J118" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
     </row>
     <row r="119" spans="1:10" x14ac:dyDescent="0.2">
@@ -23676,7 +23634,7 @@
         <v>62</v>
       </c>
       <c r="J119" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
     </row>
     <row r="120" spans="1:10" x14ac:dyDescent="0.2">
@@ -23728,7 +23686,7 @@
         <v>62</v>
       </c>
       <c r="J121" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
     </row>
     <row r="122" spans="1:10" x14ac:dyDescent="0.2">
@@ -23754,7 +23712,7 @@
         <v>62</v>
       </c>
       <c r="J122" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
     </row>
     <row r="123" spans="1:10" x14ac:dyDescent="0.2">
@@ -23780,7 +23738,7 @@
         <v>62</v>
       </c>
       <c r="J123" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
     </row>
     <row r="124" spans="1:10" x14ac:dyDescent="0.2">
@@ -24151,10 +24109,10 @@
         <v>13</v>
       </c>
       <c r="J139" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="L139" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
     </row>
     <row r="140" spans="1:12" x14ac:dyDescent="0.2">
@@ -24180,7 +24138,7 @@
         <v>58</v>
       </c>
       <c r="J140" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
     </row>
     <row r="141" spans="1:12" x14ac:dyDescent="0.2">
@@ -24252,7 +24210,7 @@
         <v>58</v>
       </c>
       <c r="J143" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
     </row>
     <row r="144" spans="1:12" x14ac:dyDescent="0.2">
@@ -24278,7 +24236,7 @@
         <v>58</v>
       </c>
       <c r="J144" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
     </row>
     <row r="145" spans="1:10" x14ac:dyDescent="0.2">
@@ -24300,14 +24258,11 @@
       <c r="F145">
         <v>0</v>
       </c>
-      <c r="G145" t="s">
-        <v>188</v>
-      </c>
       <c r="H145" t="s">
         <v>58</v>
       </c>
       <c r="J145" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
     </row>
     <row r="146" spans="1:10" x14ac:dyDescent="0.2">
@@ -24333,7 +24288,7 @@
         <v>58</v>
       </c>
       <c r="J146" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
     </row>
     <row r="147" spans="1:10" x14ac:dyDescent="0.2">
@@ -24359,7 +24314,7 @@
         <v>62</v>
       </c>
       <c r="J147" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
     </row>
     <row r="148" spans="1:10" x14ac:dyDescent="0.2">
@@ -24385,7 +24340,7 @@
         <v>58</v>
       </c>
       <c r="J148" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
     </row>
     <row r="149" spans="1:10" x14ac:dyDescent="0.2">
@@ -24434,7 +24389,7 @@
         <v>58</v>
       </c>
       <c r="J150" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
     </row>
     <row r="151" spans="1:10" x14ac:dyDescent="0.2">
@@ -24483,7 +24438,7 @@
         <v>62</v>
       </c>
       <c r="J152" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
     </row>
     <row r="153" spans="1:10" x14ac:dyDescent="0.2">
@@ -24509,7 +24464,7 @@
         <v>58</v>
       </c>
       <c r="J153" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
     </row>
     <row r="154" spans="1:10" x14ac:dyDescent="0.2">
@@ -24673,7 +24628,7 @@
         <v>58</v>
       </c>
       <c r="J160" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="161" spans="1:10" x14ac:dyDescent="0.2">
@@ -24699,7 +24654,7 @@
         <v>62</v>
       </c>
       <c r="J161" t="s">
-        <v>225</v>
+        <v>219</v>
       </c>
     </row>
     <row r="162" spans="1:10" x14ac:dyDescent="0.2">
@@ -24725,7 +24680,7 @@
         <v>62</v>
       </c>
       <c r="J162" t="s">
-        <v>224</v>
+        <v>218</v>
       </c>
     </row>
     <row r="163" spans="1:10" x14ac:dyDescent="0.2">
@@ -24751,7 +24706,7 @@
         <v>62</v>
       </c>
       <c r="J163" t="s">
-        <v>224</v>
+        <v>218</v>
       </c>
     </row>
     <row r="164" spans="1:10" x14ac:dyDescent="0.2">
@@ -24777,7 +24732,7 @@
         <v>62</v>
       </c>
       <c r="J164" t="s">
-        <v>224</v>
+        <v>218</v>
       </c>
     </row>
     <row r="165" spans="1:10" x14ac:dyDescent="0.2">
@@ -24803,7 +24758,7 @@
         <v>62</v>
       </c>
       <c r="J165" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
     </row>
     <row r="166" spans="1:10" x14ac:dyDescent="0.2">
@@ -24829,7 +24784,7 @@
         <v>62</v>
       </c>
       <c r="J166" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
     </row>
     <row r="167" spans="1:10" x14ac:dyDescent="0.2">
@@ -24855,7 +24810,7 @@
         <v>62</v>
       </c>
       <c r="J167" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
     </row>
     <row r="168" spans="1:10" x14ac:dyDescent="0.2">
@@ -24881,7 +24836,7 @@
         <v>62</v>
       </c>
       <c r="J168" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
     </row>
     <row r="169" spans="1:10" x14ac:dyDescent="0.2">
@@ -24907,7 +24862,7 @@
         <v>62</v>
       </c>
       <c r="J169" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
     </row>
     <row r="170" spans="1:10" x14ac:dyDescent="0.2">
@@ -24933,7 +24888,7 @@
         <v>62</v>
       </c>
       <c r="J170" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
     </row>
     <row r="171" spans="1:10" x14ac:dyDescent="0.2">
@@ -24959,7 +24914,7 @@
         <v>62</v>
       </c>
       <c r="J171" t="s">
-        <v>227</v>
+        <v>221</v>
       </c>
     </row>
     <row r="172" spans="1:10" x14ac:dyDescent="0.2">
@@ -24985,7 +24940,7 @@
         <v>62</v>
       </c>
       <c r="J172" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
     </row>
     <row r="173" spans="1:10" x14ac:dyDescent="0.2">
@@ -25011,7 +24966,7 @@
         <v>62</v>
       </c>
       <c r="J173" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
     </row>
     <row r="174" spans="1:10" x14ac:dyDescent="0.2">
@@ -25037,7 +24992,7 @@
         <v>62</v>
       </c>
       <c r="J174" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
     </row>
     <row r="175" spans="1:10" x14ac:dyDescent="0.2">
@@ -25063,7 +25018,7 @@
         <v>62</v>
       </c>
       <c r="J175" t="s">
-        <v>228</v>
+        <v>222</v>
       </c>
     </row>
     <row r="176" spans="1:10" x14ac:dyDescent="0.2">
@@ -25089,7 +25044,7 @@
         <v>62</v>
       </c>
       <c r="J176" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
     </row>
     <row r="177" spans="1:10" x14ac:dyDescent="0.2">
@@ -25115,7 +25070,7 @@
         <v>62</v>
       </c>
       <c r="J177" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
     </row>
     <row r="178" spans="1:10" x14ac:dyDescent="0.2">
@@ -25141,7 +25096,7 @@
         <v>62</v>
       </c>
       <c r="J178" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
     </row>
     <row r="179" spans="1:10" x14ac:dyDescent="0.2">
@@ -25167,7 +25122,7 @@
         <v>62</v>
       </c>
       <c r="J179" t="s">
-        <v>231</v>
+        <v>225</v>
       </c>
     </row>
     <row r="180" spans="1:10" x14ac:dyDescent="0.2">
@@ -25193,7 +25148,7 @@
         <v>62</v>
       </c>
       <c r="J180" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
     </row>
     <row r="181" spans="1:10" x14ac:dyDescent="0.2">
@@ -25219,7 +25174,7 @@
         <v>62</v>
       </c>
       <c r="J181" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
     </row>
     <row r="182" spans="1:10" x14ac:dyDescent="0.2">
@@ -25245,7 +25200,7 @@
         <v>62</v>
       </c>
       <c r="J182" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
     </row>
     <row r="183" spans="1:10" x14ac:dyDescent="0.2">
@@ -25271,7 +25226,7 @@
         <v>62</v>
       </c>
       <c r="J183" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
     </row>
     <row r="184" spans="1:10" x14ac:dyDescent="0.2">
@@ -25297,7 +25252,7 @@
         <v>62</v>
       </c>
       <c r="J184" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
     </row>
     <row r="185" spans="1:10" x14ac:dyDescent="0.2">
@@ -25864,7 +25819,7 @@
         <v>13</v>
       </c>
       <c r="J208" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
     </row>
     <row r="209" spans="1:10" x14ac:dyDescent="0.2">
@@ -25890,7 +25845,7 @@
         <v>58</v>
       </c>
       <c r="J209" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
     </row>
     <row r="210" spans="1:10" x14ac:dyDescent="0.2">
@@ -25916,7 +25871,7 @@
         <v>62</v>
       </c>
       <c r="J210" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
     </row>
     <row r="211" spans="1:10" x14ac:dyDescent="0.2">
@@ -25942,7 +25897,7 @@
         <v>58</v>
       </c>
       <c r="J211" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
     </row>
     <row r="212" spans="1:10" x14ac:dyDescent="0.2">
@@ -25991,7 +25946,7 @@
         <v>13</v>
       </c>
       <c r="J213" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
     </row>
     <row r="214" spans="1:10" x14ac:dyDescent="0.2">
@@ -26017,7 +25972,7 @@
         <v>58</v>
       </c>
       <c r="J214" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
     </row>
     <row r="215" spans="1:10" x14ac:dyDescent="0.2">
@@ -26043,7 +25998,7 @@
         <v>13</v>
       </c>
       <c r="J215" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
     </row>
     <row r="216" spans="1:10" x14ac:dyDescent="0.2">
@@ -26161,7 +26116,7 @@
         <v>13</v>
       </c>
       <c r="J220" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
     </row>
     <row r="221" spans="1:10" x14ac:dyDescent="0.2">
@@ -26187,7 +26142,7 @@
         <v>62</v>
       </c>
       <c r="J221" t="s">
-        <v>233</v>
+        <v>227</v>
       </c>
     </row>
     <row r="222" spans="1:10" x14ac:dyDescent="0.2">
@@ -26213,7 +26168,7 @@
         <v>62</v>
       </c>
       <c r="J222" t="s">
-        <v>233</v>
+        <v>227</v>
       </c>
     </row>
     <row r="223" spans="1:10" x14ac:dyDescent="0.2">
@@ -26239,7 +26194,7 @@
         <v>62</v>
       </c>
       <c r="J223" t="s">
-        <v>234</v>
+        <v>228</v>
       </c>
     </row>
     <row r="224" spans="1:10" x14ac:dyDescent="0.2">
@@ -26265,7 +26220,7 @@
         <v>62</v>
       </c>
       <c r="J224" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
     </row>
     <row r="225" spans="1:10" x14ac:dyDescent="0.2">
@@ -26291,7 +26246,7 @@
         <v>62</v>
       </c>
       <c r="J225" t="s">
-        <v>233</v>
+        <v>227</v>
       </c>
     </row>
     <row r="226" spans="1:10" x14ac:dyDescent="0.2">
@@ -26317,7 +26272,7 @@
         <v>62</v>
       </c>
       <c r="J226" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
     </row>
     <row r="227" spans="1:10" x14ac:dyDescent="0.2">
@@ -26343,7 +26298,7 @@
         <v>62</v>
       </c>
       <c r="J227" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
     </row>
     <row r="228" spans="1:10" x14ac:dyDescent="0.2">
@@ -26369,7 +26324,7 @@
         <v>62</v>
       </c>
       <c r="J228" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
     </row>
     <row r="229" spans="1:10" x14ac:dyDescent="0.2">
@@ -26395,7 +26350,7 @@
         <v>62</v>
       </c>
       <c r="J229" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
     </row>
     <row r="230" spans="1:10" x14ac:dyDescent="0.2">
@@ -26421,7 +26376,7 @@
         <v>62</v>
       </c>
       <c r="J230" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
     </row>
     <row r="231" spans="1:10" x14ac:dyDescent="0.2">
@@ -26447,7 +26402,7 @@
         <v>62</v>
       </c>
       <c r="J231" t="s">
-        <v>236</v>
+        <v>230</v>
       </c>
     </row>
     <row r="232" spans="1:10" x14ac:dyDescent="0.2">
@@ -26473,7 +26428,7 @@
         <v>62</v>
       </c>
       <c r="J232" t="s">
-        <v>236</v>
+        <v>230</v>
       </c>
     </row>
     <row r="233" spans="1:10" x14ac:dyDescent="0.2">
@@ -26499,7 +26454,7 @@
         <v>62</v>
       </c>
       <c r="J233" t="s">
-        <v>236</v>
+        <v>230</v>
       </c>
     </row>
     <row r="234" spans="1:10" x14ac:dyDescent="0.2">
@@ -26525,7 +26480,7 @@
         <v>62</v>
       </c>
       <c r="J234" t="s">
-        <v>237</v>
+        <v>231</v>
       </c>
     </row>
     <row r="235" spans="1:10" x14ac:dyDescent="0.2">
@@ -26551,7 +26506,7 @@
         <v>62</v>
       </c>
       <c r="J235" t="s">
-        <v>239</v>
+        <v>233</v>
       </c>
     </row>
     <row r="236" spans="1:10" x14ac:dyDescent="0.2">
@@ -26577,7 +26532,7 @@
         <v>62</v>
       </c>
       <c r="J236" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
     </row>
     <row r="237" spans="1:10" x14ac:dyDescent="0.2">
@@ -26603,7 +26558,7 @@
         <v>62</v>
       </c>
       <c r="J237" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
     </row>
     <row r="238" spans="1:10" x14ac:dyDescent="0.2">
@@ -26629,7 +26584,7 @@
         <v>62</v>
       </c>
       <c r="J238" t="s">
-        <v>241</v>
+        <v>235</v>
       </c>
     </row>
     <row r="239" spans="1:10" x14ac:dyDescent="0.2">
@@ -26655,7 +26610,7 @@
         <v>62</v>
       </c>
       <c r="J239" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
     </row>
     <row r="240" spans="1:10" x14ac:dyDescent="0.2">
@@ -26681,7 +26636,7 @@
         <v>62</v>
       </c>
       <c r="J240" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
     </row>
     <row r="241" spans="1:10" x14ac:dyDescent="0.2">
@@ -26707,7 +26662,7 @@
         <v>58</v>
       </c>
       <c r="J241" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
     </row>
     <row r="242" spans="1:10" x14ac:dyDescent="0.2">
@@ -26733,7 +26688,7 @@
         <v>58</v>
       </c>
       <c r="J242" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
     </row>
     <row r="243" spans="1:10" x14ac:dyDescent="0.2">
@@ -26759,7 +26714,7 @@
         <v>58</v>
       </c>
       <c r="J243" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
     </row>
     <row r="244" spans="1:10" x14ac:dyDescent="0.2">
@@ -26785,7 +26740,7 @@
         <v>58</v>
       </c>
       <c r="J244" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
     </row>
     <row r="245" spans="1:10" x14ac:dyDescent="0.2">
@@ -26811,7 +26766,7 @@
         <v>58</v>
       </c>
       <c r="J245" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
     </row>
     <row r="246" spans="1:10" x14ac:dyDescent="0.2">
@@ -27113,7 +27068,7 @@
         <v>56</v>
       </c>
       <c r="J258" t="s">
-        <v>243</v>
+        <v>237</v>
       </c>
     </row>
     <row r="259" spans="1:10" x14ac:dyDescent="0.2">
@@ -27231,7 +27186,7 @@
         <v>13</v>
       </c>
       <c r="J263" t="s">
-        <v>262</v>
+        <v>254</v>
       </c>
     </row>
     <row r="264" spans="1:10" x14ac:dyDescent="0.2">
@@ -27257,7 +27212,7 @@
         <v>13</v>
       </c>
       <c r="J264" t="s">
-        <v>263</v>
+        <v>255</v>
       </c>
     </row>
     <row r="265" spans="1:10" x14ac:dyDescent="0.2">
@@ -27306,7 +27261,7 @@
         <v>58</v>
       </c>
       <c r="J266" t="s">
-        <v>264</v>
+        <v>256</v>
       </c>
     </row>
     <row r="267" spans="1:10" x14ac:dyDescent="0.2">
@@ -27328,14 +27283,11 @@
       <c r="F267">
         <v>0</v>
       </c>
-      <c r="G267" t="s">
-        <v>265</v>
-      </c>
       <c r="H267" t="s">
         <v>58</v>
       </c>
       <c r="J267" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
     </row>
     <row r="268" spans="1:10" x14ac:dyDescent="0.2">
@@ -27407,7 +27359,7 @@
         <v>62</v>
       </c>
       <c r="J270" t="s">
-        <v>267</v>
+        <v>258</v>
       </c>
     </row>
     <row r="271" spans="1:10" x14ac:dyDescent="0.2">
@@ -27433,7 +27385,7 @@
         <v>58</v>
       </c>
       <c r="J271" t="s">
-        <v>268</v>
+        <v>259</v>
       </c>
     </row>
     <row r="272" spans="1:10" x14ac:dyDescent="0.2">
@@ -27459,7 +27411,7 @@
         <v>58</v>
       </c>
       <c r="J272" t="s">
-        <v>268</v>
+        <v>259</v>
       </c>
     </row>
     <row r="273" spans="1:10" x14ac:dyDescent="0.2">
@@ -27485,7 +27437,7 @@
         <v>58</v>
       </c>
       <c r="J273" t="s">
-        <v>268</v>
+        <v>259</v>
       </c>
     </row>
     <row r="274" spans="1:10" x14ac:dyDescent="0.2">
@@ -27511,7 +27463,7 @@
         <v>58</v>
       </c>
       <c r="J274" t="s">
-        <v>268</v>
+        <v>259</v>
       </c>
     </row>
     <row r="275" spans="1:10" x14ac:dyDescent="0.2">
@@ -27537,7 +27489,7 @@
         <v>13</v>
       </c>
       <c r="J275" t="s">
-        <v>269</v>
+        <v>260</v>
       </c>
     </row>
     <row r="276" spans="1:10" x14ac:dyDescent="0.2">
@@ -27655,7 +27607,7 @@
         <v>58</v>
       </c>
       <c r="J280" t="s">
-        <v>308</v>
+        <v>298</v>
       </c>
     </row>
     <row r="281" spans="1:10" x14ac:dyDescent="0.2">
@@ -27681,7 +27633,7 @@
         <v>62</v>
       </c>
       <c r="J281" t="s">
-        <v>309</v>
+        <v>299</v>
       </c>
     </row>
     <row r="282" spans="1:10" x14ac:dyDescent="0.2">
@@ -27707,7 +27659,7 @@
         <v>62</v>
       </c>
       <c r="J282" t="s">
-        <v>311</v>
+        <v>301</v>
       </c>
     </row>
     <row r="283" spans="1:10" x14ac:dyDescent="0.2">
@@ -27733,7 +27685,7 @@
         <v>62</v>
       </c>
       <c r="J283" t="s">
-        <v>312</v>
+        <v>302</v>
       </c>
     </row>
     <row r="284" spans="1:10" x14ac:dyDescent="0.2">
@@ -27759,7 +27711,7 @@
         <v>62</v>
       </c>
       <c r="J284" t="s">
-        <v>313</v>
+        <v>303</v>
       </c>
     </row>
     <row r="285" spans="1:10" x14ac:dyDescent="0.2">
@@ -27785,7 +27737,7 @@
         <v>62</v>
       </c>
       <c r="J285" t="s">
-        <v>312</v>
+        <v>302</v>
       </c>
     </row>
     <row r="286" spans="1:10" x14ac:dyDescent="0.2">
@@ -27811,7 +27763,7 @@
         <v>62</v>
       </c>
       <c r="J286" t="s">
-        <v>313</v>
+        <v>303</v>
       </c>
     </row>
     <row r="287" spans="1:10" x14ac:dyDescent="0.2">
@@ -27837,7 +27789,7 @@
         <v>62</v>
       </c>
       <c r="J287" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
     </row>
     <row r="288" spans="1:10" x14ac:dyDescent="0.2">
@@ -27863,7 +27815,7 @@
         <v>62</v>
       </c>
       <c r="J288" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
     </row>
     <row r="289" spans="1:10" x14ac:dyDescent="0.2">
@@ -27889,7 +27841,7 @@
         <v>62</v>
       </c>
       <c r="J289" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
     </row>
     <row r="290" spans="1:10" x14ac:dyDescent="0.2">
@@ -27915,7 +27867,7 @@
         <v>62</v>
       </c>
       <c r="J290" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
     </row>
     <row r="291" spans="1:10" x14ac:dyDescent="0.2">
@@ -27941,7 +27893,7 @@
         <v>62</v>
       </c>
       <c r="J291" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
     </row>
     <row r="292" spans="1:10" x14ac:dyDescent="0.2">
@@ -27967,7 +27919,7 @@
         <v>62</v>
       </c>
       <c r="J292" t="s">
-        <v>314</v>
+        <v>304</v>
       </c>
     </row>
     <row r="293" spans="1:10" x14ac:dyDescent="0.2">
@@ -27993,7 +27945,7 @@
         <v>62</v>
       </c>
       <c r="J293" t="s">
-        <v>315</v>
+        <v>305</v>
       </c>
     </row>
     <row r="294" spans="1:10" x14ac:dyDescent="0.2">
@@ -28019,7 +27971,7 @@
         <v>62</v>
       </c>
       <c r="J294" t="s">
-        <v>316</v>
+        <v>306</v>
       </c>
     </row>
     <row r="295" spans="1:10" x14ac:dyDescent="0.2">
@@ -28045,7 +27997,7 @@
         <v>62</v>
       </c>
       <c r="J295" t="s">
-        <v>314</v>
+        <v>304</v>
       </c>
     </row>
     <row r="296" spans="1:10" x14ac:dyDescent="0.2">
@@ -28071,7 +28023,7 @@
         <v>62</v>
       </c>
       <c r="J296" t="s">
-        <v>314</v>
+        <v>304</v>
       </c>
     </row>
     <row r="297" spans="1:10" x14ac:dyDescent="0.2">
@@ -28097,7 +28049,7 @@
         <v>62</v>
       </c>
       <c r="J297" t="s">
-        <v>317</v>
+        <v>307</v>
       </c>
     </row>
     <row r="298" spans="1:10" x14ac:dyDescent="0.2">
@@ -28123,7 +28075,7 @@
         <v>62</v>
       </c>
       <c r="J298" t="s">
-        <v>317</v>
+        <v>307</v>
       </c>
     </row>
     <row r="299" spans="1:10" x14ac:dyDescent="0.2">
@@ -28149,7 +28101,7 @@
         <v>62</v>
       </c>
       <c r="J299" t="s">
-        <v>317</v>
+        <v>307</v>
       </c>
     </row>
     <row r="300" spans="1:10" x14ac:dyDescent="0.2">
@@ -28175,7 +28127,7 @@
         <v>58</v>
       </c>
       <c r="J300" t="s">
-        <v>318</v>
+        <v>308</v>
       </c>
     </row>
     <row r="301" spans="1:10" x14ac:dyDescent="0.2">
@@ -28201,7 +28153,7 @@
         <v>62</v>
       </c>
       <c r="J301" t="s">
-        <v>317</v>
+        <v>307</v>
       </c>
     </row>
     <row r="302" spans="1:10" x14ac:dyDescent="0.2">
@@ -28227,7 +28179,7 @@
         <v>62</v>
       </c>
       <c r="J302" t="s">
-        <v>319</v>
+        <v>309</v>
       </c>
     </row>
     <row r="303" spans="1:10" x14ac:dyDescent="0.2">
@@ -28253,7 +28205,7 @@
         <v>62</v>
       </c>
       <c r="J303" t="s">
-        <v>319</v>
+        <v>309</v>
       </c>
     </row>
     <row r="304" spans="1:10" x14ac:dyDescent="0.2">
@@ -28279,7 +28231,7 @@
         <v>62</v>
       </c>
       <c r="J304" t="s">
-        <v>319</v>
+        <v>309</v>
       </c>
     </row>
     <row r="305" spans="1:10" x14ac:dyDescent="0.2">
@@ -28305,7 +28257,7 @@
         <v>62</v>
       </c>
       <c r="J305" t="s">
-        <v>320</v>
+        <v>310</v>
       </c>
     </row>
     <row r="306" spans="1:10" x14ac:dyDescent="0.2">
@@ -28331,7 +28283,7 @@
         <v>62</v>
       </c>
       <c r="J306" t="s">
-        <v>319</v>
+        <v>309</v>
       </c>
     </row>
     <row r="307" spans="1:10" x14ac:dyDescent="0.2">
@@ -28426,7 +28378,7 @@
         <v>58</v>
       </c>
       <c r="J310" t="s">
-        <v>244</v>
+        <v>238</v>
       </c>
     </row>
     <row r="311" spans="1:10" x14ac:dyDescent="0.2">
@@ -28659,7 +28611,7 @@
         <v>58</v>
       </c>
       <c r="J320" t="s">
-        <v>245</v>
+        <v>239</v>
       </c>
     </row>
     <row r="321" spans="1:10" x14ac:dyDescent="0.2">
@@ -28731,7 +28683,7 @@
         <v>62</v>
       </c>
       <c r="J323" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
     </row>
     <row r="324" spans="1:10" x14ac:dyDescent="0.2">
@@ -28757,7 +28709,7 @@
         <v>13</v>
       </c>
       <c r="J324" t="s">
-        <v>270</v>
+        <v>261</v>
       </c>
     </row>
     <row r="325" spans="1:10" x14ac:dyDescent="0.2">
@@ -28783,7 +28735,7 @@
         <v>59</v>
       </c>
       <c r="J325" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
     </row>
     <row r="326" spans="1:10" x14ac:dyDescent="0.2">
@@ -28809,7 +28761,7 @@
         <v>59</v>
       </c>
       <c r="J326" t="s">
-        <v>273</v>
+        <v>264</v>
       </c>
     </row>
     <row r="327" spans="1:10" x14ac:dyDescent="0.2">
@@ -28831,14 +28783,11 @@
       <c r="F327">
         <v>0</v>
       </c>
-      <c r="G327" t="s">
+      <c r="H327" t="s">
+        <v>62</v>
+      </c>
+      <c r="J327" t="s">
         <v>265</v>
-      </c>
-      <c r="H327" t="s">
-        <v>62</v>
-      </c>
-      <c r="J327" t="s">
-        <v>274</v>
       </c>
     </row>
     <row r="328" spans="1:10" x14ac:dyDescent="0.2">
@@ -28864,7 +28813,7 @@
         <v>58</v>
       </c>
       <c r="J328" t="s">
-        <v>275</v>
+        <v>266</v>
       </c>
     </row>
     <row r="329" spans="1:10" x14ac:dyDescent="0.2">
@@ -28890,7 +28839,7 @@
         <v>58</v>
       </c>
       <c r="J329" t="s">
-        <v>275</v>
+        <v>266</v>
       </c>
     </row>
     <row r="330" spans="1:10" x14ac:dyDescent="0.2">
@@ -28916,7 +28865,7 @@
         <v>58</v>
       </c>
       <c r="J330" t="s">
-        <v>276</v>
+        <v>267</v>
       </c>
     </row>
     <row r="331" spans="1:10" x14ac:dyDescent="0.2">
@@ -28942,7 +28891,7 @@
         <v>13</v>
       </c>
       <c r="J331" t="s">
-        <v>277</v>
+        <v>268</v>
       </c>
     </row>
     <row r="332" spans="1:10" x14ac:dyDescent="0.2">
@@ -28968,7 +28917,7 @@
         <v>59</v>
       </c>
       <c r="J332" t="s">
-        <v>278</v>
+        <v>269</v>
       </c>
     </row>
     <row r="333" spans="1:10" x14ac:dyDescent="0.2">
@@ -28994,7 +28943,7 @@
         <v>58</v>
       </c>
       <c r="J333" t="s">
-        <v>275</v>
+        <v>266</v>
       </c>
     </row>
     <row r="334" spans="1:10" x14ac:dyDescent="0.2">
@@ -29020,7 +28969,7 @@
         <v>13</v>
       </c>
       <c r="J334" t="s">
-        <v>279</v>
+        <v>270</v>
       </c>
     </row>
     <row r="335" spans="1:10" x14ac:dyDescent="0.2">
@@ -29046,7 +28995,7 @@
         <v>58</v>
       </c>
       <c r="J335" t="s">
-        <v>275</v>
+        <v>266</v>
       </c>
     </row>
     <row r="336" spans="1:10" x14ac:dyDescent="0.2">
@@ -29233,7 +29182,7 @@
         <v>62</v>
       </c>
       <c r="J343" t="s">
-        <v>321</v>
+        <v>311</v>
       </c>
     </row>
     <row r="344" spans="1:10" x14ac:dyDescent="0.2">
@@ -29259,7 +29208,7 @@
         <v>58</v>
       </c>
       <c r="J344" t="s">
-        <v>322</v>
+        <v>312</v>
       </c>
     </row>
     <row r="345" spans="1:10" x14ac:dyDescent="0.2">
@@ -29285,7 +29234,7 @@
         <v>62</v>
       </c>
       <c r="J345" t="s">
-        <v>323</v>
+        <v>313</v>
       </c>
     </row>
     <row r="346" spans="1:10" x14ac:dyDescent="0.2">
@@ -29311,7 +29260,7 @@
         <v>62</v>
       </c>
       <c r="J346" t="s">
-        <v>323</v>
+        <v>313</v>
       </c>
     </row>
     <row r="347" spans="1:10" x14ac:dyDescent="0.2">
@@ -29337,7 +29286,7 @@
         <v>62</v>
       </c>
       <c r="J347" t="s">
-        <v>323</v>
+        <v>313</v>
       </c>
     </row>
     <row r="348" spans="1:10" x14ac:dyDescent="0.2">
@@ -29363,7 +29312,7 @@
         <v>62</v>
       </c>
       <c r="J348" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
     </row>
     <row r="349" spans="1:10" x14ac:dyDescent="0.2">
@@ -29389,7 +29338,7 @@
         <v>62</v>
       </c>
       <c r="J349" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
     </row>
     <row r="350" spans="1:10" x14ac:dyDescent="0.2">
@@ -29415,7 +29364,7 @@
         <v>62</v>
       </c>
       <c r="J350" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
     </row>
     <row r="351" spans="1:10" x14ac:dyDescent="0.2">
@@ -29441,7 +29390,7 @@
         <v>62</v>
       </c>
       <c r="J351" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
     </row>
     <row r="352" spans="1:10" x14ac:dyDescent="0.2">
@@ -29467,7 +29416,7 @@
         <v>62</v>
       </c>
       <c r="J352" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
     </row>
     <row r="353" spans="1:10" x14ac:dyDescent="0.2">
@@ -29493,7 +29442,7 @@
         <v>58</v>
       </c>
       <c r="J353" t="s">
-        <v>324</v>
+        <v>314</v>
       </c>
     </row>
     <row r="354" spans="1:10" x14ac:dyDescent="0.2">
@@ -29519,7 +29468,7 @@
         <v>58</v>
       </c>
       <c r="J354" t="s">
-        <v>325</v>
+        <v>315</v>
       </c>
     </row>
     <row r="355" spans="1:10" x14ac:dyDescent="0.2">
@@ -29545,7 +29494,7 @@
         <v>62</v>
       </c>
       <c r="J355" t="s">
-        <v>316</v>
+        <v>306</v>
       </c>
     </row>
     <row r="356" spans="1:10" x14ac:dyDescent="0.2">
@@ -29571,7 +29520,7 @@
         <v>62</v>
       </c>
       <c r="J356" t="s">
-        <v>314</v>
+        <v>304</v>
       </c>
     </row>
     <row r="357" spans="1:10" x14ac:dyDescent="0.2">
@@ -29597,7 +29546,7 @@
         <v>56</v>
       </c>
       <c r="J357" t="s">
-        <v>326</v>
+        <v>316</v>
       </c>
     </row>
     <row r="358" spans="1:10" x14ac:dyDescent="0.2">
@@ -29623,7 +29572,7 @@
         <v>62</v>
       </c>
       <c r="J358" t="s">
-        <v>317</v>
+        <v>307</v>
       </c>
     </row>
     <row r="359" spans="1:10" x14ac:dyDescent="0.2">
@@ -29645,14 +29594,11 @@
       <c r="F359">
         <v>0</v>
       </c>
-      <c r="G359" t="s">
-        <v>331</v>
-      </c>
       <c r="H359" t="s">
         <v>62</v>
       </c>
       <c r="J359" t="s">
-        <v>317</v>
+        <v>307</v>
       </c>
     </row>
     <row r="360" spans="1:10" x14ac:dyDescent="0.2">
@@ -29678,7 +29624,7 @@
         <v>62</v>
       </c>
       <c r="J360" t="s">
-        <v>327</v>
+        <v>317</v>
       </c>
     </row>
     <row r="361" spans="1:10" x14ac:dyDescent="0.2">
@@ -29704,7 +29650,7 @@
         <v>58</v>
       </c>
       <c r="J361" t="s">
-        <v>328</v>
+        <v>318</v>
       </c>
     </row>
     <row r="362" spans="1:10" x14ac:dyDescent="0.2">
@@ -29730,7 +29676,7 @@
         <v>62</v>
       </c>
       <c r="J362" t="s">
-        <v>329</v>
+        <v>319</v>
       </c>
     </row>
     <row r="363" spans="1:10" x14ac:dyDescent="0.2">
@@ -29756,7 +29702,7 @@
         <v>62</v>
       </c>
       <c r="J363" t="s">
-        <v>330</v>
+        <v>320</v>
       </c>
     </row>
     <row r="364" spans="1:10" x14ac:dyDescent="0.2">
@@ -29782,7 +29728,7 @@
         <v>58</v>
       </c>
       <c r="J364" t="s">
-        <v>333</v>
+        <v>322</v>
       </c>
     </row>
     <row r="365" spans="1:10" x14ac:dyDescent="0.2">
@@ -29808,7 +29754,7 @@
         <v>58</v>
       </c>
       <c r="J365" t="s">
-        <v>333</v>
+        <v>322</v>
       </c>
     </row>
     <row r="366" spans="1:10" x14ac:dyDescent="0.2">
@@ -29834,7 +29780,7 @@
         <v>62</v>
       </c>
       <c r="J366" t="s">
-        <v>332</v>
+        <v>321</v>
       </c>
     </row>
     <row r="367" spans="1:10" x14ac:dyDescent="0.2">
@@ -29860,7 +29806,7 @@
         <v>58</v>
       </c>
       <c r="J367" t="s">
-        <v>333</v>
+        <v>322</v>
       </c>
     </row>
     <row r="368" spans="1:10" x14ac:dyDescent="0.2">
@@ -30231,7 +30177,7 @@
         <v>58</v>
       </c>
       <c r="J383" t="s">
-        <v>280</v>
+        <v>271</v>
       </c>
     </row>
     <row r="384" spans="1:10" x14ac:dyDescent="0.2">
@@ -30280,7 +30226,7 @@
         <v>13</v>
       </c>
       <c r="J385" t="s">
-        <v>281</v>
+        <v>272</v>
       </c>
     </row>
     <row r="386" spans="1:10" x14ac:dyDescent="0.2">
@@ -30398,7 +30344,7 @@
         <v>58</v>
       </c>
       <c r="J390" t="s">
-        <v>282</v>
+        <v>273</v>
       </c>
     </row>
     <row r="391" spans="1:10" x14ac:dyDescent="0.2">
@@ -30723,7 +30669,7 @@
         <v>62</v>
       </c>
       <c r="J404" t="s">
-        <v>334</v>
+        <v>323</v>
       </c>
     </row>
     <row r="405" spans="1:10" x14ac:dyDescent="0.2">
@@ -30749,7 +30695,7 @@
         <v>62</v>
       </c>
       <c r="J405" t="s">
-        <v>335</v>
+        <v>324</v>
       </c>
     </row>
     <row r="406" spans="1:10" x14ac:dyDescent="0.2">
@@ -30775,7 +30721,7 @@
         <v>62</v>
       </c>
       <c r="J406" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
     </row>
     <row r="407" spans="1:10" x14ac:dyDescent="0.2">
@@ -30801,7 +30747,7 @@
         <v>62</v>
       </c>
       <c r="J407" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
     </row>
     <row r="408" spans="1:10" x14ac:dyDescent="0.2">
@@ -30827,7 +30773,7 @@
         <v>62</v>
       </c>
       <c r="J408" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
     </row>
     <row r="409" spans="1:10" x14ac:dyDescent="0.2">
@@ -30983,7 +30929,7 @@
         <v>62</v>
       </c>
       <c r="J414" t="s">
-        <v>296</v>
+        <v>286</v>
       </c>
     </row>
     <row r="415" spans="1:10" x14ac:dyDescent="0.2">
@@ -31009,7 +30955,7 @@
         <v>62</v>
       </c>
       <c r="J415" t="s">
-        <v>337</v>
+        <v>326</v>
       </c>
     </row>
     <row r="416" spans="1:10" x14ac:dyDescent="0.2">
@@ -31035,7 +30981,7 @@
         <v>62</v>
       </c>
       <c r="J416" t="s">
-        <v>336</v>
+        <v>325</v>
       </c>
     </row>
     <row r="417" spans="1:10" x14ac:dyDescent="0.2">
@@ -31061,7 +31007,7 @@
         <v>62</v>
       </c>
       <c r="J417" t="s">
-        <v>339</v>
+        <v>328</v>
       </c>
     </row>
     <row r="418" spans="1:10" x14ac:dyDescent="0.2">
@@ -31087,7 +31033,7 @@
         <v>62</v>
       </c>
       <c r="J418" t="s">
-        <v>338</v>
+        <v>327</v>
       </c>
     </row>
     <row r="419" spans="1:10" x14ac:dyDescent="0.2">
@@ -31113,7 +31059,7 @@
         <v>62</v>
       </c>
       <c r="J419" t="s">
-        <v>340</v>
+        <v>329</v>
       </c>
     </row>
     <row r="420" spans="1:10" x14ac:dyDescent="0.2">
@@ -31139,7 +31085,7 @@
         <v>62</v>
       </c>
       <c r="J420" t="s">
-        <v>341</v>
+        <v>330</v>
       </c>
     </row>
     <row r="421" spans="1:10" x14ac:dyDescent="0.2">
@@ -31165,7 +31111,7 @@
         <v>62</v>
       </c>
       <c r="J421" t="s">
-        <v>342</v>
+        <v>331</v>
       </c>
     </row>
     <row r="422" spans="1:10" x14ac:dyDescent="0.2">
@@ -31191,7 +31137,7 @@
         <v>62</v>
       </c>
       <c r="J422" t="s">
-        <v>343</v>
+        <v>332</v>
       </c>
     </row>
     <row r="423" spans="1:10" x14ac:dyDescent="0.2">
@@ -31217,7 +31163,7 @@
         <v>62</v>
       </c>
       <c r="J423" t="s">
-        <v>344</v>
+        <v>333</v>
       </c>
     </row>
     <row r="424" spans="1:10" x14ac:dyDescent="0.2">
@@ -31243,7 +31189,7 @@
         <v>58</v>
       </c>
       <c r="J424" t="s">
-        <v>345</v>
+        <v>334</v>
       </c>
     </row>
     <row r="425" spans="1:10" x14ac:dyDescent="0.2">
@@ -31269,7 +31215,7 @@
         <v>58</v>
       </c>
       <c r="J425" t="s">
-        <v>346</v>
+        <v>335</v>
       </c>
     </row>
     <row r="426" spans="1:10" x14ac:dyDescent="0.2">
@@ -31295,7 +31241,7 @@
         <v>62</v>
       </c>
       <c r="J426" t="s">
-        <v>347</v>
+        <v>336</v>
       </c>
     </row>
     <row r="427" spans="1:10" x14ac:dyDescent="0.2">
@@ -31321,7 +31267,7 @@
         <v>62</v>
       </c>
       <c r="J427" t="s">
-        <v>348</v>
+        <v>337</v>
       </c>
     </row>
     <row r="428" spans="1:10" x14ac:dyDescent="0.2">
@@ -31343,14 +31289,11 @@
       <c r="F428">
         <v>0</v>
       </c>
-      <c r="G428" t="s">
-        <v>265</v>
-      </c>
       <c r="H428" t="s">
         <v>58</v>
       </c>
       <c r="J428" t="s">
-        <v>346</v>
+        <v>335</v>
       </c>
     </row>
     <row r="429" spans="1:10" x14ac:dyDescent="0.2">
@@ -31882,7 +31825,7 @@
         <v>58</v>
       </c>
       <c r="J451" t="s">
-        <v>283</v>
+        <v>274</v>
       </c>
     </row>
     <row r="452" spans="1:10" x14ac:dyDescent="0.2">
@@ -31908,7 +31851,7 @@
         <v>58</v>
       </c>
       <c r="J452" t="s">
-        <v>284</v>
+        <v>275</v>
       </c>
     </row>
     <row r="453" spans="1:10" x14ac:dyDescent="0.2">
@@ -31980,7 +31923,7 @@
         <v>58</v>
       </c>
       <c r="J455" t="s">
-        <v>283</v>
+        <v>274</v>
       </c>
     </row>
     <row r="456" spans="1:10" x14ac:dyDescent="0.2">
@@ -32029,7 +31972,7 @@
         <v>13</v>
       </c>
       <c r="J457" t="s">
-        <v>285</v>
+        <v>276</v>
       </c>
     </row>
     <row r="458" spans="1:10" x14ac:dyDescent="0.2">
@@ -32166,9 +32109,6 @@
       <c r="F463">
         <v>1</v>
       </c>
-      <c r="G463" t="s">
-        <v>286</v>
-      </c>
       <c r="H463" t="s">
         <v>13</v>
       </c>
@@ -32192,9 +32132,6 @@
       <c r="F464">
         <v>1</v>
       </c>
-      <c r="G464" t="s">
-        <v>286</v>
-      </c>
       <c r="H464" t="s">
         <v>13</v>
       </c>
@@ -32222,7 +32159,7 @@
         <v>62</v>
       </c>
       <c r="J465" t="s">
-        <v>349</v>
+        <v>338</v>
       </c>
     </row>
     <row r="466" spans="1:10" x14ac:dyDescent="0.2">
@@ -32248,7 +32185,7 @@
         <v>62</v>
       </c>
       <c r="J466" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
     </row>
     <row r="467" spans="1:10" x14ac:dyDescent="0.2">
@@ -32300,7 +32237,7 @@
         <v>62</v>
       </c>
       <c r="J468" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
     </row>
     <row r="469" spans="1:10" x14ac:dyDescent="0.2">
@@ -32326,7 +32263,7 @@
         <v>62</v>
       </c>
       <c r="J469" t="s">
-        <v>352</v>
+        <v>341</v>
       </c>
     </row>
     <row r="470" spans="1:10" x14ac:dyDescent="0.2">
@@ -32348,14 +32285,11 @@
       <c r="F470">
         <v>0</v>
       </c>
-      <c r="G470" t="s">
-        <v>353</v>
-      </c>
       <c r="H470" t="s">
         <v>62</v>
       </c>
       <c r="J470" t="s">
-        <v>205</v>
+        <v>376</v>
       </c>
     </row>
     <row r="471" spans="1:10" x14ac:dyDescent="0.2">
@@ -32381,7 +32315,7 @@
         <v>62</v>
       </c>
       <c r="J471" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
     </row>
     <row r="472" spans="1:10" x14ac:dyDescent="0.2">
@@ -32407,7 +32341,7 @@
         <v>62</v>
       </c>
       <c r="J472" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
     </row>
     <row r="473" spans="1:10" x14ac:dyDescent="0.2">
@@ -32433,7 +32367,7 @@
         <v>62</v>
       </c>
       <c r="J473" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
     </row>
     <row r="474" spans="1:10" x14ac:dyDescent="0.2">
@@ -32459,7 +32393,7 @@
         <v>62</v>
       </c>
       <c r="J474" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
     </row>
     <row r="475" spans="1:10" x14ac:dyDescent="0.2">
@@ -32485,7 +32419,7 @@
         <v>62</v>
       </c>
       <c r="J475" t="s">
-        <v>296</v>
+        <v>286</v>
       </c>
     </row>
     <row r="476" spans="1:10" x14ac:dyDescent="0.2">
@@ -32511,7 +32445,7 @@
         <v>62</v>
       </c>
       <c r="J476" t="s">
-        <v>354</v>
+        <v>342</v>
       </c>
     </row>
     <row r="477" spans="1:10" x14ac:dyDescent="0.2">
@@ -32537,7 +32471,7 @@
         <v>62</v>
       </c>
       <c r="J477" t="s">
-        <v>355</v>
+        <v>343</v>
       </c>
     </row>
     <row r="478" spans="1:10" x14ac:dyDescent="0.2">
@@ -32563,7 +32497,7 @@
         <v>62</v>
       </c>
       <c r="J478" t="s">
-        <v>356</v>
+        <v>344</v>
       </c>
     </row>
     <row r="479" spans="1:10" x14ac:dyDescent="0.2">
@@ -32589,7 +32523,7 @@
         <v>62</v>
       </c>
       <c r="J479" t="s">
-        <v>354</v>
+        <v>342</v>
       </c>
     </row>
     <row r="480" spans="1:10" x14ac:dyDescent="0.2">
@@ -32615,7 +32549,7 @@
         <v>58</v>
       </c>
       <c r="J480" t="s">
-        <v>357</v>
+        <v>345</v>
       </c>
     </row>
     <row r="481" spans="1:11" x14ac:dyDescent="0.2">
@@ -32664,7 +32598,7 @@
         <v>62</v>
       </c>
       <c r="J482" t="s">
-        <v>358</v>
+        <v>346</v>
       </c>
     </row>
     <row r="483" spans="1:11" x14ac:dyDescent="0.2">
@@ -32713,7 +32647,7 @@
         <v>62</v>
       </c>
       <c r="J484" t="s">
-        <v>359</v>
+        <v>347</v>
       </c>
     </row>
     <row r="485" spans="1:11" x14ac:dyDescent="0.2">
@@ -32739,7 +32673,7 @@
         <v>58</v>
       </c>
       <c r="J485" t="s">
-        <v>360</v>
+        <v>348</v>
       </c>
     </row>
     <row r="486" spans="1:11" x14ac:dyDescent="0.2">
@@ -32765,7 +32699,7 @@
         <v>58</v>
       </c>
       <c r="J486" t="s">
-        <v>360</v>
+        <v>348</v>
       </c>
     </row>
     <row r="487" spans="1:11" x14ac:dyDescent="0.2">
@@ -32791,7 +32725,7 @@
         <v>58</v>
       </c>
       <c r="J487" t="s">
-        <v>361</v>
+        <v>349</v>
       </c>
     </row>
     <row r="488" spans="1:11" x14ac:dyDescent="0.2">
@@ -32817,7 +32751,7 @@
         <v>62</v>
       </c>
       <c r="J488" t="s">
-        <v>362</v>
+        <v>350</v>
       </c>
     </row>
     <row r="489" spans="1:11" x14ac:dyDescent="0.2">
@@ -32843,7 +32777,7 @@
         <v>58</v>
       </c>
       <c r="J489" t="s">
-        <v>360</v>
+        <v>348</v>
       </c>
     </row>
     <row r="490" spans="1:11" x14ac:dyDescent="0.2">
@@ -32869,7 +32803,7 @@
         <v>13</v>
       </c>
       <c r="K490" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
     </row>
     <row r="491" spans="1:11" x14ac:dyDescent="0.2">
@@ -32918,7 +32852,7 @@
         <v>58</v>
       </c>
       <c r="J492" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="493" spans="1:11" x14ac:dyDescent="0.2">
@@ -32967,7 +32901,7 @@
         <v>58</v>
       </c>
       <c r="J494" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
     </row>
     <row r="495" spans="1:11" x14ac:dyDescent="0.2">
@@ -32989,14 +32923,11 @@
       <c r="F495">
         <v>0</v>
       </c>
-      <c r="G495" t="s">
-        <v>250</v>
-      </c>
       <c r="H495" t="s">
         <v>62</v>
       </c>
       <c r="J495" t="s">
-        <v>249</v>
+        <v>243</v>
       </c>
     </row>
     <row r="496" spans="1:11" x14ac:dyDescent="0.2">
@@ -33022,7 +32953,7 @@
         <v>58</v>
       </c>
       <c r="J496" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
     </row>
     <row r="497" spans="1:10" x14ac:dyDescent="0.2">
@@ -33071,7 +33002,7 @@
         <v>58</v>
       </c>
       <c r="J498" t="s">
-        <v>252</v>
+        <v>245</v>
       </c>
     </row>
     <row r="499" spans="1:10" x14ac:dyDescent="0.2">
@@ -33189,7 +33120,7 @@
         <v>58</v>
       </c>
       <c r="J503" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
     </row>
     <row r="504" spans="1:10" x14ac:dyDescent="0.2">
@@ -33238,7 +33169,7 @@
         <v>62</v>
       </c>
       <c r="J505" t="s">
-        <v>288</v>
+        <v>278</v>
       </c>
     </row>
     <row r="506" spans="1:10" x14ac:dyDescent="0.2">
@@ -33264,7 +33195,7 @@
         <v>62</v>
       </c>
       <c r="J506" t="s">
-        <v>287</v>
+        <v>277</v>
       </c>
     </row>
     <row r="507" spans="1:10" x14ac:dyDescent="0.2">
@@ -33290,7 +33221,7 @@
         <v>62</v>
       </c>
       <c r="J507" t="s">
-        <v>289</v>
+        <v>279</v>
       </c>
     </row>
     <row r="508" spans="1:10" x14ac:dyDescent="0.2">
@@ -33316,7 +33247,7 @@
         <v>62</v>
       </c>
       <c r="J508" t="s">
-        <v>290</v>
+        <v>280</v>
       </c>
     </row>
     <row r="509" spans="1:10" x14ac:dyDescent="0.2">
@@ -33342,7 +33273,7 @@
         <v>62</v>
       </c>
       <c r="J509" t="s">
-        <v>290</v>
+        <v>280</v>
       </c>
     </row>
     <row r="510" spans="1:10" x14ac:dyDescent="0.2">
@@ -33368,7 +33299,7 @@
         <v>62</v>
       </c>
       <c r="J510" t="s">
-        <v>291</v>
+        <v>281</v>
       </c>
     </row>
     <row r="511" spans="1:10" x14ac:dyDescent="0.2">
@@ -33394,7 +33325,7 @@
         <v>62</v>
       </c>
       <c r="J511" t="s">
-        <v>292</v>
+        <v>282</v>
       </c>
     </row>
     <row r="512" spans="1:10" x14ac:dyDescent="0.2">
@@ -33420,7 +33351,7 @@
         <v>62</v>
       </c>
       <c r="J512" t="s">
-        <v>293</v>
+        <v>283</v>
       </c>
     </row>
     <row r="513" spans="1:10" x14ac:dyDescent="0.2">
@@ -33442,14 +33373,11 @@
       <c r="F513">
         <v>0</v>
       </c>
-      <c r="G513" t="s">
-        <v>265</v>
-      </c>
       <c r="H513" t="s">
         <v>58</v>
       </c>
       <c r="J513" t="s">
-        <v>294</v>
+        <v>374</v>
       </c>
     </row>
     <row r="514" spans="1:10" x14ac:dyDescent="0.2">
@@ -33475,7 +33403,7 @@
         <v>58</v>
       </c>
       <c r="J514" t="s">
-        <v>294</v>
+        <v>284</v>
       </c>
     </row>
     <row r="515" spans="1:10" x14ac:dyDescent="0.2">
@@ -33501,7 +33429,7 @@
         <v>62</v>
       </c>
       <c r="J515" t="s">
-        <v>295</v>
+        <v>285</v>
       </c>
     </row>
     <row r="516" spans="1:10" x14ac:dyDescent="0.2">
@@ -33527,7 +33455,7 @@
         <v>62</v>
       </c>
       <c r="J516" t="s">
-        <v>296</v>
+        <v>286</v>
       </c>
     </row>
     <row r="517" spans="1:10" x14ac:dyDescent="0.2">
@@ -33549,14 +33477,11 @@
       <c r="F517">
         <v>0</v>
       </c>
-      <c r="G517" t="s">
-        <v>257</v>
-      </c>
       <c r="H517" t="s">
         <v>62</v>
       </c>
       <c r="J517" t="s">
-        <v>295</v>
+        <v>285</v>
       </c>
     </row>
     <row r="518" spans="1:10" x14ac:dyDescent="0.2">
@@ -33582,7 +33507,7 @@
         <v>62</v>
       </c>
       <c r="J518" t="s">
-        <v>297</v>
+        <v>287</v>
       </c>
     </row>
     <row r="519" spans="1:10" x14ac:dyDescent="0.2">
@@ -33654,7 +33579,7 @@
         <v>58</v>
       </c>
       <c r="J521" t="s">
-        <v>310</v>
+        <v>300</v>
       </c>
     </row>
     <row r="522" spans="1:10" x14ac:dyDescent="0.2">
@@ -33772,7 +33697,7 @@
         <v>62</v>
       </c>
       <c r="J526" t="s">
-        <v>363</v>
+        <v>351</v>
       </c>
     </row>
     <row r="527" spans="1:10" x14ac:dyDescent="0.2">
@@ -33798,7 +33723,7 @@
         <v>62</v>
       </c>
       <c r="J527" t="s">
-        <v>364</v>
+        <v>352</v>
       </c>
     </row>
     <row r="528" spans="1:10" x14ac:dyDescent="0.2">
@@ -33824,7 +33749,7 @@
         <v>62</v>
       </c>
       <c r="J528" t="s">
-        <v>365</v>
+        <v>353</v>
       </c>
     </row>
     <row r="529" spans="1:10" x14ac:dyDescent="0.2">
@@ -33850,7 +33775,7 @@
         <v>62</v>
       </c>
       <c r="J529" t="s">
-        <v>366</v>
+        <v>354</v>
       </c>
     </row>
     <row r="530" spans="1:10" x14ac:dyDescent="0.2">
@@ -33876,7 +33801,7 @@
         <v>62</v>
       </c>
       <c r="J530" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
     </row>
     <row r="531" spans="1:10" x14ac:dyDescent="0.2">
@@ -33902,7 +33827,7 @@
         <v>62</v>
       </c>
       <c r="J531" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
     </row>
     <row r="532" spans="1:10" x14ac:dyDescent="0.2">
@@ -33928,7 +33853,7 @@
         <v>62</v>
       </c>
       <c r="J532" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
     </row>
     <row r="533" spans="1:10" x14ac:dyDescent="0.2">
@@ -33954,7 +33879,7 @@
         <v>62</v>
       </c>
       <c r="J533" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
     </row>
     <row r="534" spans="1:10" x14ac:dyDescent="0.2">
@@ -33980,7 +33905,7 @@
         <v>62</v>
       </c>
       <c r="J534" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
     </row>
     <row r="535" spans="1:10" x14ac:dyDescent="0.2">
@@ -34006,7 +33931,7 @@
         <v>62</v>
       </c>
       <c r="J535" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
     </row>
     <row r="536" spans="1:10" x14ac:dyDescent="0.2">
@@ -34032,7 +33957,7 @@
         <v>62</v>
       </c>
       <c r="J536" t="s">
-        <v>367</v>
+        <v>355</v>
       </c>
     </row>
     <row r="537" spans="1:10" x14ac:dyDescent="0.2">
@@ -34058,7 +33983,7 @@
         <v>62</v>
       </c>
       <c r="J537" t="s">
-        <v>367</v>
+        <v>355</v>
       </c>
     </row>
     <row r="538" spans="1:10" x14ac:dyDescent="0.2">
@@ -34084,7 +34009,7 @@
         <v>62</v>
       </c>
       <c r="J538" t="s">
-        <v>368</v>
+        <v>356</v>
       </c>
     </row>
     <row r="539" spans="1:10" x14ac:dyDescent="0.2">
@@ -34110,7 +34035,7 @@
         <v>62</v>
       </c>
       <c r="J539" t="s">
-        <v>369</v>
+        <v>357</v>
       </c>
     </row>
     <row r="540" spans="1:10" x14ac:dyDescent="0.2">
@@ -34136,7 +34061,7 @@
         <v>62</v>
       </c>
       <c r="J540" t="s">
-        <v>370</v>
+        <v>358</v>
       </c>
     </row>
     <row r="541" spans="1:10" x14ac:dyDescent="0.2">
@@ -34162,7 +34087,7 @@
         <v>62</v>
       </c>
       <c r="J541" t="s">
-        <v>371</v>
+        <v>359</v>
       </c>
     </row>
     <row r="542" spans="1:10" x14ac:dyDescent="0.2">
@@ -34188,7 +34113,7 @@
         <v>62</v>
       </c>
       <c r="J542" t="s">
-        <v>371</v>
+        <v>359</v>
       </c>
     </row>
     <row r="543" spans="1:10" x14ac:dyDescent="0.2">
@@ -34214,7 +34139,7 @@
         <v>62</v>
       </c>
       <c r="J543" t="s">
-        <v>371</v>
+        <v>359</v>
       </c>
     </row>
     <row r="544" spans="1:10" x14ac:dyDescent="0.2">
@@ -34266,7 +34191,7 @@
         <v>62</v>
       </c>
       <c r="J545" t="s">
-        <v>371</v>
+        <v>359</v>
       </c>
     </row>
     <row r="546" spans="1:10" x14ac:dyDescent="0.2">
@@ -34318,7 +34243,7 @@
         <v>62</v>
       </c>
       <c r="J547" t="s">
-        <v>372</v>
+        <v>360</v>
       </c>
     </row>
     <row r="548" spans="1:10" x14ac:dyDescent="0.2">
@@ -34344,7 +34269,7 @@
         <v>62</v>
       </c>
       <c r="J548" t="s">
-        <v>372</v>
+        <v>360</v>
       </c>
     </row>
     <row r="549" spans="1:10" x14ac:dyDescent="0.2">
@@ -34370,7 +34295,7 @@
         <v>58</v>
       </c>
       <c r="J549" t="s">
-        <v>373</v>
+        <v>361</v>
       </c>
     </row>
     <row r="550" spans="1:10" x14ac:dyDescent="0.2">
@@ -34422,7 +34347,7 @@
         <v>58</v>
       </c>
       <c r="J551" t="s">
-        <v>256</v>
+        <v>249</v>
       </c>
     </row>
     <row r="552" spans="1:10" x14ac:dyDescent="0.2">
@@ -34448,7 +34373,7 @@
         <v>58</v>
       </c>
       <c r="J552" t="s">
-        <v>256</v>
+        <v>249</v>
       </c>
     </row>
     <row r="553" spans="1:10" x14ac:dyDescent="0.2">
@@ -34474,7 +34399,7 @@
         <v>58</v>
       </c>
       <c r="J553" t="s">
-        <v>254</v>
+        <v>247</v>
       </c>
     </row>
     <row r="554" spans="1:10" x14ac:dyDescent="0.2">
@@ -34615,7 +34540,7 @@
         <v>58</v>
       </c>
       <c r="J559" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
     </row>
     <row r="560" spans="1:10" x14ac:dyDescent="0.2">
@@ -34637,14 +34562,11 @@
       <c r="F560">
         <v>0</v>
       </c>
-      <c r="G560" t="s">
-        <v>257</v>
-      </c>
       <c r="H560" t="s">
         <v>62</v>
       </c>
       <c r="J560" t="s">
-        <v>258</v>
+        <v>250</v>
       </c>
     </row>
     <row r="561" spans="1:10" x14ac:dyDescent="0.2">
@@ -34689,14 +34611,11 @@
       <c r="F562">
         <v>0</v>
       </c>
-      <c r="G562" t="s">
-        <v>257</v>
-      </c>
       <c r="H562" t="s">
         <v>62</v>
       </c>
       <c r="J562" t="s">
-        <v>259</v>
+        <v>251</v>
       </c>
     </row>
     <row r="563" spans="1:10" x14ac:dyDescent="0.2">
@@ -34745,7 +34664,7 @@
         <v>13</v>
       </c>
       <c r="J564" t="s">
-        <v>260</v>
+        <v>252</v>
       </c>
     </row>
     <row r="565" spans="1:10" x14ac:dyDescent="0.2">
@@ -34771,7 +34690,7 @@
         <v>58</v>
       </c>
       <c r="J565" t="s">
-        <v>261</v>
+        <v>253</v>
       </c>
     </row>
     <row r="566" spans="1:10" x14ac:dyDescent="0.2">
@@ -34797,7 +34716,7 @@
         <v>62</v>
       </c>
       <c r="J566" t="s">
-        <v>298</v>
+        <v>288</v>
       </c>
     </row>
     <row r="567" spans="1:10" x14ac:dyDescent="0.2">
@@ -34823,7 +34742,7 @@
         <v>58</v>
       </c>
       <c r="J567" t="s">
-        <v>299</v>
+        <v>289</v>
       </c>
     </row>
     <row r="568" spans="1:10" x14ac:dyDescent="0.2">
@@ -34849,7 +34768,7 @@
         <v>62</v>
       </c>
       <c r="J568" t="s">
-        <v>296</v>
+        <v>286</v>
       </c>
     </row>
     <row r="569" spans="1:10" x14ac:dyDescent="0.2">
@@ -34875,7 +34794,7 @@
         <v>58</v>
       </c>
       <c r="J569" t="s">
-        <v>300</v>
+        <v>290</v>
       </c>
     </row>
     <row r="570" spans="1:10" x14ac:dyDescent="0.2">
@@ -34901,7 +34820,7 @@
         <v>62</v>
       </c>
       <c r="J570" t="s">
-        <v>301</v>
+        <v>291</v>
       </c>
     </row>
     <row r="571" spans="1:10" x14ac:dyDescent="0.2">
@@ -34927,7 +34846,7 @@
         <v>62</v>
       </c>
       <c r="J571" t="s">
-        <v>301</v>
+        <v>291</v>
       </c>
     </row>
     <row r="572" spans="1:10" x14ac:dyDescent="0.2">
@@ -34953,7 +34872,7 @@
         <v>62</v>
       </c>
       <c r="J572" t="s">
-        <v>302</v>
+        <v>292</v>
       </c>
     </row>
     <row r="573" spans="1:10" x14ac:dyDescent="0.2">
@@ -34979,7 +34898,7 @@
         <v>58</v>
       </c>
       <c r="J573" t="s">
-        <v>303</v>
+        <v>293</v>
       </c>
     </row>
     <row r="574" spans="1:10" x14ac:dyDescent="0.2">
@@ -35005,7 +34924,7 @@
         <v>58</v>
       </c>
       <c r="J574" t="s">
-        <v>304</v>
+        <v>294</v>
       </c>
     </row>
     <row r="575" spans="1:10" x14ac:dyDescent="0.2">
@@ -35054,7 +34973,7 @@
         <v>62</v>
       </c>
       <c r="J576" t="s">
-        <v>307</v>
+        <v>297</v>
       </c>
     </row>
     <row r="577" spans="1:10" x14ac:dyDescent="0.2">
@@ -35076,14 +34995,11 @@
       <c r="F577">
         <v>0</v>
       </c>
-      <c r="G577" t="s">
-        <v>257</v>
-      </c>
       <c r="H577" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="J577" t="s">
-        <v>305</v>
+        <v>375</v>
       </c>
     </row>
     <row r="578" spans="1:10" x14ac:dyDescent="0.2">
@@ -35105,14 +35021,11 @@
       <c r="F578">
         <v>0</v>
       </c>
-      <c r="G578" t="s">
-        <v>257</v>
-      </c>
       <c r="H578" t="s">
         <v>62</v>
       </c>
       <c r="J578" t="s">
-        <v>305</v>
+        <v>295</v>
       </c>
     </row>
     <row r="579" spans="1:10" x14ac:dyDescent="0.2">
@@ -35134,14 +35047,11 @@
       <c r="F579">
         <v>0</v>
       </c>
-      <c r="G579" t="s">
-        <v>265</v>
-      </c>
       <c r="H579" t="s">
         <v>58</v>
       </c>
       <c r="J579" t="s">
-        <v>306</v>
+        <v>296</v>
       </c>
     </row>
     <row r="580" spans="1:10" x14ac:dyDescent="0.2">
@@ -35167,7 +35077,7 @@
         <v>62</v>
       </c>
       <c r="J580" t="s">
-        <v>307</v>
+        <v>297</v>
       </c>
     </row>
     <row r="581" spans="1:10" x14ac:dyDescent="0.2">
@@ -35331,7 +35241,7 @@
         <v>62</v>
       </c>
       <c r="J587" t="s">
-        <v>374</v>
+        <v>362</v>
       </c>
     </row>
     <row r="588" spans="1:10" x14ac:dyDescent="0.2">
@@ -35357,7 +35267,7 @@
         <v>62</v>
       </c>
       <c r="J588" t="s">
-        <v>375</v>
+        <v>363</v>
       </c>
     </row>
     <row r="589" spans="1:10" x14ac:dyDescent="0.2">
@@ -35383,7 +35293,7 @@
         <v>62</v>
       </c>
       <c r="J589" t="s">
-        <v>375</v>
+        <v>363</v>
       </c>
     </row>
     <row r="590" spans="1:10" x14ac:dyDescent="0.2">
@@ -35409,7 +35319,7 @@
         <v>62</v>
       </c>
       <c r="J590" t="s">
-        <v>376</v>
+        <v>364</v>
       </c>
     </row>
     <row r="591" spans="1:10" x14ac:dyDescent="0.2">
@@ -35435,7 +35345,7 @@
         <v>62</v>
       </c>
       <c r="J591" t="s">
-        <v>376</v>
+        <v>364</v>
       </c>
     </row>
     <row r="592" spans="1:10" x14ac:dyDescent="0.2">
@@ -35461,7 +35371,7 @@
         <v>62</v>
       </c>
       <c r="J592" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
     </row>
     <row r="593" spans="1:10" x14ac:dyDescent="0.2">
@@ -35487,7 +35397,7 @@
         <v>62</v>
       </c>
       <c r="J593" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
     </row>
     <row r="594" spans="1:10" x14ac:dyDescent="0.2">
@@ -35513,7 +35423,7 @@
         <v>62</v>
       </c>
       <c r="J594" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
     </row>
     <row r="595" spans="1:10" x14ac:dyDescent="0.2">
@@ -35539,7 +35449,7 @@
         <v>62</v>
       </c>
       <c r="J595" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
     </row>
     <row r="596" spans="1:10" x14ac:dyDescent="0.2">
@@ -35565,7 +35475,7 @@
         <v>62</v>
       </c>
       <c r="J596" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
     </row>
     <row r="597" spans="1:10" x14ac:dyDescent="0.2">
@@ -35591,7 +35501,7 @@
         <v>62</v>
       </c>
       <c r="J597" t="s">
-        <v>377</v>
+        <v>365</v>
       </c>
     </row>
     <row r="598" spans="1:10" x14ac:dyDescent="0.2">
@@ -35617,7 +35527,7 @@
         <v>62</v>
       </c>
       <c r="J598" t="s">
-        <v>377</v>
+        <v>365</v>
       </c>
     </row>
     <row r="599" spans="1:10" x14ac:dyDescent="0.2">
@@ -35643,7 +35553,7 @@
         <v>62</v>
       </c>
       <c r="J599" t="s">
-        <v>378</v>
+        <v>366</v>
       </c>
     </row>
     <row r="600" spans="1:10" x14ac:dyDescent="0.2">
@@ -35669,7 +35579,7 @@
         <v>62</v>
       </c>
       <c r="J600" t="s">
-        <v>377</v>
+        <v>365</v>
       </c>
     </row>
     <row r="601" spans="1:10" x14ac:dyDescent="0.2">
@@ -35695,7 +35605,7 @@
         <v>62</v>
       </c>
       <c r="J601" t="s">
-        <v>337</v>
+        <v>326</v>
       </c>
     </row>
     <row r="602" spans="1:10" x14ac:dyDescent="0.2">
@@ -35721,7 +35631,7 @@
         <v>62</v>
       </c>
       <c r="J602" t="s">
-        <v>379</v>
+        <v>367</v>
       </c>
     </row>
     <row r="603" spans="1:10" x14ac:dyDescent="0.2">
@@ -35747,7 +35657,7 @@
         <v>62</v>
       </c>
       <c r="J603" t="s">
-        <v>379</v>
+        <v>367</v>
       </c>
     </row>
     <row r="604" spans="1:10" x14ac:dyDescent="0.2">
@@ -35773,7 +35683,7 @@
         <v>62</v>
       </c>
       <c r="J604" t="s">
-        <v>380</v>
+        <v>368</v>
       </c>
     </row>
     <row r="605" spans="1:10" x14ac:dyDescent="0.2">
@@ -35799,7 +35709,7 @@
         <v>59</v>
       </c>
       <c r="J605" t="s">
-        <v>381</v>
+        <v>369</v>
       </c>
     </row>
     <row r="606" spans="1:10" x14ac:dyDescent="0.2">
@@ -35825,7 +35735,7 @@
         <v>62</v>
       </c>
       <c r="J606" t="s">
-        <v>379</v>
+        <v>367</v>
       </c>
     </row>
     <row r="607" spans="1:10" x14ac:dyDescent="0.2">
@@ -35851,7 +35761,7 @@
         <v>58</v>
       </c>
       <c r="J607" t="s">
-        <v>382</v>
+        <v>370</v>
       </c>
     </row>
     <row r="608" spans="1:10" x14ac:dyDescent="0.2">
@@ -35903,7 +35813,7 @@
         <v>62</v>
       </c>
       <c r="J609" t="s">
-        <v>383</v>
+        <v>371</v>
       </c>
     </row>
     <row r="610" spans="1:10" x14ac:dyDescent="0.2">
@@ -35929,7 +35839,7 @@
         <v>62</v>
       </c>
       <c r="J610" t="s">
-        <v>384</v>
+        <v>372</v>
       </c>
     </row>
     <row r="611" spans="1:10" x14ac:dyDescent="0.2">
@@ -35955,7 +35865,7 @@
         <v>62</v>
       </c>
       <c r="J611" t="s">
-        <v>385</v>
+        <v>373</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Density sweep follow-up, updated code, protocol, readme etc.
</commit_message>
<xml_diff>
--- a/documents/results_raw_two_seeds.xlsx
+++ b/documents/results_raw_two_seeds.xlsx
@@ -1,23 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10917"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Nagc2/Desktop/so101-vla-data-study/documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA1062B2-B25B-4745-BC16-0A6CD7E9AE07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{279AD80F-FF60-324B-B70B-FB9FF58AD620}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16720" yWindow="720" windowWidth="17120" windowHeight="20180" activeTab="2" xr2:uid="{E9882473-D8D3-4249-9541-943B7997CA3D}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="17120" windowHeight="20180" activeTab="3" xr2:uid="{E9882473-D8D3-4249-9541-943B7997CA3D}"/>
   </bookViews>
   <sheets>
     <sheet name="results" sheetId="1" r:id="rId1"/>
     <sheet name="exploratory results" sheetId="3" r:id="rId2"/>
     <sheet name="density_sweep" sheetId="6" r:id="rId3"/>
-    <sheet name="failure mode options" sheetId="2" r:id="rId4"/>
-    <sheet name="bench_check" sheetId="5" r:id="rId5"/>
+    <sheet name="density_followup" sheetId="7" r:id="rId4"/>
+    <sheet name="failure mode options" sheetId="2" r:id="rId5"/>
+    <sheet name="bench_check" sheetId="5" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">results!$A$1:$K$301</definedName>
@@ -68,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6625" uniqueCount="377">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7093" uniqueCount="430">
   <si>
     <t>condition</t>
   </si>
@@ -1199,6 +1200,165 @@
   </si>
   <si>
     <t>went to t1, cup started 1 inch higher than the position it should be in</t>
+  </si>
+  <si>
+    <t>in_distribution_rebuilt</t>
+  </si>
+  <si>
+    <t>aimed left and bumped cube while opening</t>
+  </si>
+  <si>
+    <t>Missed the cup, dropped the cube to the right of it, went towards fallend cube but didn't get it</t>
+  </si>
+  <si>
+    <t>Missed the cup, dropped the cube to the right of it by around an inch, went towards fallend cube but fifn't get it</t>
+  </si>
+  <si>
+    <t>opened on the top of the cube but didn't touch it</t>
+  </si>
+  <si>
+    <t>had cube in the middle of the cup, but pulled a bit back and dropped</t>
+  </si>
+  <si>
+    <t>missed the cube and went to the top</t>
+  </si>
+  <si>
+    <t>looked at cube for a second before going to top</t>
+  </si>
+  <si>
+    <t>new_positions_rebuilt</t>
+  </si>
+  <si>
+    <t>Went to the middle, towards T3</t>
+  </si>
+  <si>
+    <t>went towards T2 first</t>
+  </si>
+  <si>
+    <t xml:space="preserve">went to the middle towards T4 </t>
+  </si>
+  <si>
+    <t>seemed to aim towards cube, ended near T1</t>
+  </si>
+  <si>
+    <t>seemed to aim towards cube, ended near T2, cup was shifted, confirm this was during episode</t>
+  </si>
+  <si>
+    <t>seems to aim towards cube, went to cup, bumped it, then to T2</t>
+  </si>
+  <si>
+    <t>seems to aim towards cube, went to cup, bumped it, then to T2, ends up by E1 at certain points</t>
+  </si>
+  <si>
+    <t>goes past cube, between T4 and E3, then ends up at top of board</t>
+  </si>
+  <si>
+    <t>went towards t6, then t7, ended by t3</t>
+  </si>
+  <si>
+    <t>went towards t4, over the cube, went to t3</t>
+  </si>
+  <si>
+    <t>went towards the cube, but a bit over, then to t7, and ended by the top</t>
+  </si>
+  <si>
+    <t>went towards the cube, but a bit over, then to t7</t>
+  </si>
+  <si>
+    <t>aimed towards cube but went over, then to T7</t>
+  </si>
+  <si>
+    <t>initially looked at t6 but went towards the middle, and then towards the top of the board, near T4</t>
+  </si>
+  <si>
+    <t>ended up going to the middle, by t4 and t7</t>
+  </si>
+  <si>
+    <t>went between t6 and t7, ended near the tp, by t4</t>
+  </si>
+  <si>
+    <t>went towards t7, then t4 and near the top of the board</t>
+  </si>
+  <si>
+    <t>randomized-runpod</t>
+  </si>
+  <si>
+    <t>aimed left of cube and ended towards the top of the board</t>
+  </si>
+  <si>
+    <t>went to top of cube but didn't touch the cube</t>
+  </si>
+  <si>
+    <t>aimed to the left of the cube, opened gripper and bumped it trying to catch</t>
+  </si>
+  <si>
+    <t>bumped cube trying to get it, then went to T4</t>
+  </si>
+  <si>
+    <t>aimed to the left of the cube, opened gripper and bumped it trying to grab it</t>
+  </si>
+  <si>
+    <t>went to grab it, but didn't collect it, and bumped cube</t>
+  </si>
+  <si>
+    <t>overshot the cube, slughtly bumped it then went up</t>
+  </si>
+  <si>
+    <t>aimed correctly, but missed, then went to the top</t>
+  </si>
+  <si>
+    <t>went to the middle, then slightl corrected and bumped cube a bit, then ended up at the top</t>
+  </si>
+  <si>
+    <t>slightly bumped cube as it approached it, moved it out of place and failed on the retry</t>
+  </si>
+  <si>
+    <t>went between t6 and t7, ended by t7</t>
+  </si>
+  <si>
+    <t>went between t6 and t7, ended at t7</t>
+  </si>
+  <si>
+    <t>aimed close to cube, but to the left, bumped the cube very slighly , ended at T7</t>
+  </si>
+  <si>
+    <t>aimed close to cube, but to the left, bumped the cube slighly, ended at t7</t>
+  </si>
+  <si>
+    <t>aimed close to cube, but to the left, bumped the cube, ended at t7</t>
+  </si>
+  <si>
+    <t>was aiming to the left of the cube then went to T7</t>
+  </si>
+  <si>
+    <t>reach_e5</t>
+  </si>
+  <si>
+    <t>It didn't drop cube initially, but dropped it on the edge and it fell in</t>
+  </si>
+  <si>
+    <t>was a bit too to the left, and didn't pushed cube but didn't grab it</t>
+  </si>
+  <si>
+    <t>missed the first grab, but then got it</t>
+  </si>
+  <si>
+    <t>aimed differently, closed in front of the cube bumping it</t>
+  </si>
+  <si>
+    <t>aimed differently, closed on the cube but didn't grab it</t>
+  </si>
+  <si>
+    <t>went between t6 and t7, closer to t6, but ended by t7</t>
+  </si>
+  <si>
+    <t>went towards t7, ended closer to t4</t>
+  </si>
+  <si>
+    <t>went between t7 and t4, ended near t4</t>
+  </si>
+  <si>
+    <t>went between t6 and t7, then to t7, ended near the top of the board, between t7 and t4</t>
   </si>
 </sst>
 </file>
@@ -35892,6 +36052,2483 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B54633EB-78EE-F546-B69A-B7FF584C2DB2}">
+  <dimension ref="A1:J96"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="18.6640625" customWidth="1"/>
+    <col min="2" max="2" width="33.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" t="s">
+        <v>377</v>
+      </c>
+      <c r="C2">
+        <v>1000</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="H2" t="s">
+        <v>62</v>
+      </c>
+      <c r="J2" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" t="s">
+        <v>377</v>
+      </c>
+      <c r="C3">
+        <v>1000</v>
+      </c>
+      <c r="D3">
+        <v>2</v>
+      </c>
+      <c r="E3" t="s">
+        <v>35</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+      <c r="H3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" t="s">
+        <v>377</v>
+      </c>
+      <c r="C4">
+        <v>1000</v>
+      </c>
+      <c r="D4">
+        <v>3</v>
+      </c>
+      <c r="E4" t="s">
+        <v>35</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
+      <c r="H4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" t="s">
+        <v>377</v>
+      </c>
+      <c r="C5">
+        <v>1000</v>
+      </c>
+      <c r="D5">
+        <v>4</v>
+      </c>
+      <c r="E5" t="s">
+        <v>35</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="H5" t="s">
+        <v>58</v>
+      </c>
+      <c r="J5" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" t="s">
+        <v>377</v>
+      </c>
+      <c r="C6">
+        <v>1000</v>
+      </c>
+      <c r="D6">
+        <v>5</v>
+      </c>
+      <c r="E6" t="s">
+        <v>35</v>
+      </c>
+      <c r="F6">
+        <v>0</v>
+      </c>
+      <c r="H6" t="s">
+        <v>59</v>
+      </c>
+      <c r="J6" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" t="s">
+        <v>377</v>
+      </c>
+      <c r="C7">
+        <v>1000</v>
+      </c>
+      <c r="D7">
+        <v>6</v>
+      </c>
+      <c r="E7" t="s">
+        <v>35</v>
+      </c>
+      <c r="F7">
+        <v>0</v>
+      </c>
+      <c r="H7" t="s">
+        <v>59</v>
+      </c>
+      <c r="J7" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>377</v>
+      </c>
+      <c r="C8">
+        <v>1000</v>
+      </c>
+      <c r="D8">
+        <v>7</v>
+      </c>
+      <c r="E8" t="s">
+        <v>35</v>
+      </c>
+      <c r="F8">
+        <v>0</v>
+      </c>
+      <c r="H8" t="s">
+        <v>62</v>
+      </c>
+      <c r="J8" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9" t="s">
+        <v>377</v>
+      </c>
+      <c r="C9">
+        <v>1000</v>
+      </c>
+      <c r="D9">
+        <v>8</v>
+      </c>
+      <c r="E9" t="s">
+        <v>35</v>
+      </c>
+      <c r="F9">
+        <v>0</v>
+      </c>
+      <c r="H9" t="s">
+        <v>59</v>
+      </c>
+      <c r="J9" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>7</v>
+      </c>
+      <c r="B10" t="s">
+        <v>377</v>
+      </c>
+      <c r="C10">
+        <v>1000</v>
+      </c>
+      <c r="D10">
+        <v>9</v>
+      </c>
+      <c r="E10" t="s">
+        <v>35</v>
+      </c>
+      <c r="F10">
+        <v>1</v>
+      </c>
+      <c r="H10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>7</v>
+      </c>
+      <c r="B11" t="s">
+        <v>377</v>
+      </c>
+      <c r="C11">
+        <v>1000</v>
+      </c>
+      <c r="D11">
+        <v>10</v>
+      </c>
+      <c r="E11" t="s">
+        <v>35</v>
+      </c>
+      <c r="F11">
+        <v>0</v>
+      </c>
+      <c r="H11" t="s">
+        <v>58</v>
+      </c>
+      <c r="J11" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>7</v>
+      </c>
+      <c r="B12" t="s">
+        <v>377</v>
+      </c>
+      <c r="C12">
+        <v>1000</v>
+      </c>
+      <c r="D12">
+        <v>11</v>
+      </c>
+      <c r="E12" t="s">
+        <v>35</v>
+      </c>
+      <c r="F12">
+        <v>0</v>
+      </c>
+      <c r="H12" t="s">
+        <v>62</v>
+      </c>
+      <c r="J12" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>7</v>
+      </c>
+      <c r="B13" t="s">
+        <v>377</v>
+      </c>
+      <c r="C13">
+        <v>1000</v>
+      </c>
+      <c r="D13">
+        <v>12</v>
+      </c>
+      <c r="E13" t="s">
+        <v>35</v>
+      </c>
+      <c r="F13">
+        <v>0</v>
+      </c>
+      <c r="H13" t="s">
+        <v>58</v>
+      </c>
+      <c r="J13" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>7</v>
+      </c>
+      <c r="B14" t="s">
+        <v>377</v>
+      </c>
+      <c r="C14">
+        <v>1000</v>
+      </c>
+      <c r="D14">
+        <v>13</v>
+      </c>
+      <c r="E14" t="s">
+        <v>35</v>
+      </c>
+      <c r="F14">
+        <v>0</v>
+      </c>
+      <c r="H14" t="s">
+        <v>59</v>
+      </c>
+      <c r="J14" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>7</v>
+      </c>
+      <c r="B15" t="s">
+        <v>377</v>
+      </c>
+      <c r="C15">
+        <v>1000</v>
+      </c>
+      <c r="D15">
+        <v>14</v>
+      </c>
+      <c r="E15" t="s">
+        <v>35</v>
+      </c>
+      <c r="F15">
+        <v>1</v>
+      </c>
+      <c r="H15" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>7</v>
+      </c>
+      <c r="B16" t="s">
+        <v>377</v>
+      </c>
+      <c r="C16">
+        <v>1000</v>
+      </c>
+      <c r="D16">
+        <v>15</v>
+      </c>
+      <c r="E16" t="s">
+        <v>35</v>
+      </c>
+      <c r="F16">
+        <v>0</v>
+      </c>
+      <c r="H16" t="s">
+        <v>59</v>
+      </c>
+      <c r="J16" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>7</v>
+      </c>
+      <c r="B17" t="s">
+        <v>385</v>
+      </c>
+      <c r="C17">
+        <v>1000</v>
+      </c>
+      <c r="D17">
+        <v>1</v>
+      </c>
+      <c r="E17" t="s">
+        <v>23</v>
+      </c>
+      <c r="F17">
+        <v>0</v>
+      </c>
+      <c r="H17" t="s">
+        <v>62</v>
+      </c>
+      <c r="J17" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>7</v>
+      </c>
+      <c r="B18" t="s">
+        <v>385</v>
+      </c>
+      <c r="C18">
+        <v>1000</v>
+      </c>
+      <c r="D18">
+        <v>2</v>
+      </c>
+      <c r="E18" t="s">
+        <v>23</v>
+      </c>
+      <c r="F18">
+        <v>0</v>
+      </c>
+      <c r="H18" t="s">
+        <v>62</v>
+      </c>
+      <c r="J18" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>7</v>
+      </c>
+      <c r="B19" t="s">
+        <v>385</v>
+      </c>
+      <c r="C19">
+        <v>1000</v>
+      </c>
+      <c r="D19">
+        <v>3</v>
+      </c>
+      <c r="E19" t="s">
+        <v>23</v>
+      </c>
+      <c r="F19">
+        <v>0</v>
+      </c>
+      <c r="H19" t="s">
+        <v>62</v>
+      </c>
+      <c r="J19" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>7</v>
+      </c>
+      <c r="B20" t="s">
+        <v>385</v>
+      </c>
+      <c r="C20">
+        <v>1000</v>
+      </c>
+      <c r="D20">
+        <v>4</v>
+      </c>
+      <c r="E20" t="s">
+        <v>23</v>
+      </c>
+      <c r="F20">
+        <v>0</v>
+      </c>
+      <c r="H20" t="s">
+        <v>62</v>
+      </c>
+      <c r="J20" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>7</v>
+      </c>
+      <c r="B21" t="s">
+        <v>385</v>
+      </c>
+      <c r="C21">
+        <v>1000</v>
+      </c>
+      <c r="D21">
+        <v>5</v>
+      </c>
+      <c r="E21" t="s">
+        <v>23</v>
+      </c>
+      <c r="F21">
+        <v>0</v>
+      </c>
+      <c r="H21" t="s">
+        <v>62</v>
+      </c>
+      <c r="J21" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>7</v>
+      </c>
+      <c r="B22" t="s">
+        <v>385</v>
+      </c>
+      <c r="C22">
+        <v>1000</v>
+      </c>
+      <c r="D22">
+        <v>6</v>
+      </c>
+      <c r="E22" t="s">
+        <v>24</v>
+      </c>
+      <c r="F22">
+        <v>0</v>
+      </c>
+      <c r="H22" t="s">
+        <v>62</v>
+      </c>
+      <c r="J22" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>7</v>
+      </c>
+      <c r="B23" t="s">
+        <v>385</v>
+      </c>
+      <c r="C23">
+        <v>1000</v>
+      </c>
+      <c r="D23">
+        <v>7</v>
+      </c>
+      <c r="E23" t="s">
+        <v>24</v>
+      </c>
+      <c r="F23">
+        <v>0</v>
+      </c>
+      <c r="H23" t="s">
+        <v>62</v>
+      </c>
+      <c r="J23" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>7</v>
+      </c>
+      <c r="B24" t="s">
+        <v>385</v>
+      </c>
+      <c r="C24">
+        <v>1000</v>
+      </c>
+      <c r="D24">
+        <v>8</v>
+      </c>
+      <c r="E24" t="s">
+        <v>24</v>
+      </c>
+      <c r="F24">
+        <v>0</v>
+      </c>
+      <c r="H24" t="s">
+        <v>62</v>
+      </c>
+      <c r="J24" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>7</v>
+      </c>
+      <c r="B25" t="s">
+        <v>385</v>
+      </c>
+      <c r="C25">
+        <v>1000</v>
+      </c>
+      <c r="D25">
+        <v>9</v>
+      </c>
+      <c r="E25" t="s">
+        <v>24</v>
+      </c>
+      <c r="F25">
+        <v>0</v>
+      </c>
+      <c r="H25" t="s">
+        <v>62</v>
+      </c>
+      <c r="J25" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>7</v>
+      </c>
+      <c r="B26" t="s">
+        <v>385</v>
+      </c>
+      <c r="C26">
+        <v>1000</v>
+      </c>
+      <c r="D26">
+        <v>10</v>
+      </c>
+      <c r="E26" t="s">
+        <v>24</v>
+      </c>
+      <c r="F26">
+        <v>0</v>
+      </c>
+      <c r="H26" t="s">
+        <v>62</v>
+      </c>
+      <c r="J26" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>7</v>
+      </c>
+      <c r="B27" t="s">
+        <v>385</v>
+      </c>
+      <c r="C27">
+        <v>1000</v>
+      </c>
+      <c r="D27">
+        <v>11</v>
+      </c>
+      <c r="E27" t="s">
+        <v>25</v>
+      </c>
+      <c r="F27">
+        <v>0</v>
+      </c>
+      <c r="H27" t="s">
+        <v>62</v>
+      </c>
+      <c r="J27" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>7</v>
+      </c>
+      <c r="B28" t="s">
+        <v>385</v>
+      </c>
+      <c r="C28">
+        <v>1000</v>
+      </c>
+      <c r="D28">
+        <v>12</v>
+      </c>
+      <c r="E28" t="s">
+        <v>25</v>
+      </c>
+      <c r="F28">
+        <v>0</v>
+      </c>
+      <c r="H28" t="s">
+        <v>62</v>
+      </c>
+      <c r="J28" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>7</v>
+      </c>
+      <c r="B29" t="s">
+        <v>385</v>
+      </c>
+      <c r="C29">
+        <v>1000</v>
+      </c>
+      <c r="D29">
+        <v>13</v>
+      </c>
+      <c r="E29" t="s">
+        <v>25</v>
+      </c>
+      <c r="F29">
+        <v>0</v>
+      </c>
+      <c r="H29" t="s">
+        <v>62</v>
+      </c>
+      <c r="J29" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>7</v>
+      </c>
+      <c r="B30" t="s">
+        <v>385</v>
+      </c>
+      <c r="C30">
+        <v>1000</v>
+      </c>
+      <c r="D30">
+        <v>14</v>
+      </c>
+      <c r="E30" t="s">
+        <v>25</v>
+      </c>
+      <c r="F30">
+        <v>0</v>
+      </c>
+      <c r="H30" t="s">
+        <v>62</v>
+      </c>
+      <c r="J30" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>7</v>
+      </c>
+      <c r="B31" t="s">
+        <v>385</v>
+      </c>
+      <c r="C31">
+        <v>1000</v>
+      </c>
+      <c r="D31">
+        <v>15</v>
+      </c>
+      <c r="E31" t="s">
+        <v>25</v>
+      </c>
+      <c r="F31">
+        <v>0</v>
+      </c>
+      <c r="H31" t="s">
+        <v>62</v>
+      </c>
+      <c r="J31" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>7</v>
+      </c>
+      <c r="B32" t="s">
+        <v>385</v>
+      </c>
+      <c r="C32">
+        <v>1000</v>
+      </c>
+      <c r="D32">
+        <v>16</v>
+      </c>
+      <c r="E32" t="s">
+        <v>26</v>
+      </c>
+      <c r="F32">
+        <v>0</v>
+      </c>
+      <c r="H32" t="s">
+        <v>62</v>
+      </c>
+      <c r="J32" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>7</v>
+      </c>
+      <c r="B33" t="s">
+        <v>385</v>
+      </c>
+      <c r="C33">
+        <v>1000</v>
+      </c>
+      <c r="D33">
+        <v>17</v>
+      </c>
+      <c r="E33" t="s">
+        <v>26</v>
+      </c>
+      <c r="F33">
+        <v>0</v>
+      </c>
+      <c r="H33" t="s">
+        <v>62</v>
+      </c>
+      <c r="J33" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>7</v>
+      </c>
+      <c r="B34" t="s">
+        <v>385</v>
+      </c>
+      <c r="C34">
+        <v>1000</v>
+      </c>
+      <c r="D34">
+        <v>18</v>
+      </c>
+      <c r="E34" t="s">
+        <v>26</v>
+      </c>
+      <c r="F34">
+        <v>0</v>
+      </c>
+      <c r="H34" t="s">
+        <v>62</v>
+      </c>
+      <c r="J34" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>7</v>
+      </c>
+      <c r="B35" t="s">
+        <v>385</v>
+      </c>
+      <c r="C35">
+        <v>1000</v>
+      </c>
+      <c r="D35">
+        <v>19</v>
+      </c>
+      <c r="E35" t="s">
+        <v>26</v>
+      </c>
+      <c r="F35">
+        <v>0</v>
+      </c>
+      <c r="H35" t="s">
+        <v>62</v>
+      </c>
+      <c r="J35" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>7</v>
+      </c>
+      <c r="B36" t="s">
+        <v>385</v>
+      </c>
+      <c r="C36">
+        <v>1000</v>
+      </c>
+      <c r="D36">
+        <v>20</v>
+      </c>
+      <c r="E36" t="s">
+        <v>26</v>
+      </c>
+      <c r="F36">
+        <v>0</v>
+      </c>
+      <c r="H36" t="s">
+        <v>62</v>
+      </c>
+      <c r="J36" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>7</v>
+      </c>
+      <c r="B37" t="s">
+        <v>385</v>
+      </c>
+      <c r="C37">
+        <v>1000</v>
+      </c>
+      <c r="D37">
+        <v>21</v>
+      </c>
+      <c r="E37" t="s">
+        <v>27</v>
+      </c>
+      <c r="F37">
+        <v>0</v>
+      </c>
+      <c r="H37" t="s">
+        <v>62</v>
+      </c>
+      <c r="J37" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>7</v>
+      </c>
+      <c r="B38" t="s">
+        <v>385</v>
+      </c>
+      <c r="C38">
+        <v>1000</v>
+      </c>
+      <c r="D38">
+        <v>22</v>
+      </c>
+      <c r="E38" t="s">
+        <v>27</v>
+      </c>
+      <c r="F38">
+        <v>0</v>
+      </c>
+      <c r="H38" t="s">
+        <v>62</v>
+      </c>
+      <c r="J38" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>7</v>
+      </c>
+      <c r="B39" t="s">
+        <v>385</v>
+      </c>
+      <c r="C39">
+        <v>1000</v>
+      </c>
+      <c r="D39">
+        <v>23</v>
+      </c>
+      <c r="E39" t="s">
+        <v>27</v>
+      </c>
+      <c r="F39">
+        <v>0</v>
+      </c>
+      <c r="H39" t="s">
+        <v>62</v>
+      </c>
+      <c r="J39" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>7</v>
+      </c>
+      <c r="B40" t="s">
+        <v>385</v>
+      </c>
+      <c r="C40">
+        <v>1000</v>
+      </c>
+      <c r="D40">
+        <v>24</v>
+      </c>
+      <c r="E40" t="s">
+        <v>27</v>
+      </c>
+      <c r="F40">
+        <v>0</v>
+      </c>
+      <c r="H40" t="s">
+        <v>62</v>
+      </c>
+      <c r="J40" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>7</v>
+      </c>
+      <c r="B41" t="s">
+        <v>385</v>
+      </c>
+      <c r="C41">
+        <v>1000</v>
+      </c>
+      <c r="D41">
+        <v>25</v>
+      </c>
+      <c r="E41" t="s">
+        <v>27</v>
+      </c>
+      <c r="F41">
+        <v>0</v>
+      </c>
+      <c r="H41" t="s">
+        <v>62</v>
+      </c>
+      <c r="J41" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>403</v>
+      </c>
+      <c r="B42" t="s">
+        <v>377</v>
+      </c>
+      <c r="C42">
+        <v>1000</v>
+      </c>
+      <c r="D42">
+        <v>1</v>
+      </c>
+      <c r="E42" t="s">
+        <v>35</v>
+      </c>
+      <c r="F42">
+        <v>0</v>
+      </c>
+      <c r="H42" t="s">
+        <v>62</v>
+      </c>
+      <c r="J42" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>403</v>
+      </c>
+      <c r="B43" t="s">
+        <v>377</v>
+      </c>
+      <c r="C43">
+        <v>1000</v>
+      </c>
+      <c r="D43">
+        <v>2</v>
+      </c>
+      <c r="E43" t="s">
+        <v>35</v>
+      </c>
+      <c r="F43">
+        <v>0</v>
+      </c>
+      <c r="H43" t="s">
+        <v>58</v>
+      </c>
+      <c r="J43" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>403</v>
+      </c>
+      <c r="B44" t="s">
+        <v>377</v>
+      </c>
+      <c r="C44">
+        <v>1000</v>
+      </c>
+      <c r="D44">
+        <v>3</v>
+      </c>
+      <c r="E44" t="s">
+        <v>35</v>
+      </c>
+      <c r="F44">
+        <v>0</v>
+      </c>
+      <c r="H44" t="s">
+        <v>62</v>
+      </c>
+      <c r="J44" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>403</v>
+      </c>
+      <c r="B45" t="s">
+        <v>377</v>
+      </c>
+      <c r="C45">
+        <v>1000</v>
+      </c>
+      <c r="D45">
+        <v>4</v>
+      </c>
+      <c r="E45" t="s">
+        <v>35</v>
+      </c>
+      <c r="F45">
+        <v>0</v>
+      </c>
+      <c r="H45" t="s">
+        <v>58</v>
+      </c>
+      <c r="J45" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>403</v>
+      </c>
+      <c r="B46" t="s">
+        <v>377</v>
+      </c>
+      <c r="C46">
+        <v>1000</v>
+      </c>
+      <c r="D46">
+        <v>5</v>
+      </c>
+      <c r="E46" t="s">
+        <v>35</v>
+      </c>
+      <c r="F46">
+        <v>0</v>
+      </c>
+      <c r="H46" t="s">
+        <v>58</v>
+      </c>
+      <c r="J46" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
+        <v>403</v>
+      </c>
+      <c r="B47" t="s">
+        <v>377</v>
+      </c>
+      <c r="C47">
+        <v>1000</v>
+      </c>
+      <c r="D47">
+        <v>6</v>
+      </c>
+      <c r="E47" t="s">
+        <v>35</v>
+      </c>
+      <c r="F47">
+        <v>0</v>
+      </c>
+      <c r="H47" t="s">
+        <v>58</v>
+      </c>
+      <c r="J47" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>403</v>
+      </c>
+      <c r="B48" t="s">
+        <v>377</v>
+      </c>
+      <c r="C48">
+        <v>1000</v>
+      </c>
+      <c r="D48">
+        <v>7</v>
+      </c>
+      <c r="E48" t="s">
+        <v>35</v>
+      </c>
+      <c r="F48">
+        <v>0</v>
+      </c>
+      <c r="H48" t="s">
+        <v>58</v>
+      </c>
+      <c r="J48" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>403</v>
+      </c>
+      <c r="B49" t="s">
+        <v>377</v>
+      </c>
+      <c r="C49">
+        <v>1000</v>
+      </c>
+      <c r="D49">
+        <v>8</v>
+      </c>
+      <c r="E49" t="s">
+        <v>35</v>
+      </c>
+      <c r="F49">
+        <v>0</v>
+      </c>
+      <c r="H49" t="s">
+        <v>58</v>
+      </c>
+      <c r="J49" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
+        <v>403</v>
+      </c>
+      <c r="B50" t="s">
+        <v>377</v>
+      </c>
+      <c r="C50">
+        <v>1000</v>
+      </c>
+      <c r="D50">
+        <v>9</v>
+      </c>
+      <c r="E50" t="s">
+        <v>35</v>
+      </c>
+      <c r="F50">
+        <v>0</v>
+      </c>
+      <c r="H50" t="s">
+        <v>58</v>
+      </c>
+      <c r="J50" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
+        <v>403</v>
+      </c>
+      <c r="B51" t="s">
+        <v>377</v>
+      </c>
+      <c r="C51">
+        <v>1000</v>
+      </c>
+      <c r="D51">
+        <v>10</v>
+      </c>
+      <c r="E51" t="s">
+        <v>35</v>
+      </c>
+      <c r="F51">
+        <v>1</v>
+      </c>
+      <c r="H51" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
+        <v>403</v>
+      </c>
+      <c r="B52" t="s">
+        <v>377</v>
+      </c>
+      <c r="C52">
+        <v>1000</v>
+      </c>
+      <c r="D52">
+        <v>11</v>
+      </c>
+      <c r="E52" t="s">
+        <v>35</v>
+      </c>
+      <c r="F52">
+        <v>0</v>
+      </c>
+      <c r="H52" t="s">
+        <v>58</v>
+      </c>
+      <c r="J52" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
+        <v>403</v>
+      </c>
+      <c r="B53" t="s">
+        <v>377</v>
+      </c>
+      <c r="C53">
+        <v>1000</v>
+      </c>
+      <c r="D53">
+        <v>12</v>
+      </c>
+      <c r="E53" t="s">
+        <v>35</v>
+      </c>
+      <c r="F53">
+        <v>0</v>
+      </c>
+      <c r="H53" t="s">
+        <v>58</v>
+      </c>
+      <c r="J53" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
+        <v>403</v>
+      </c>
+      <c r="B54" t="s">
+        <v>377</v>
+      </c>
+      <c r="C54">
+        <v>1000</v>
+      </c>
+      <c r="D54">
+        <v>13</v>
+      </c>
+      <c r="E54" t="s">
+        <v>35</v>
+      </c>
+      <c r="F54">
+        <v>0</v>
+      </c>
+      <c r="H54" t="s">
+        <v>58</v>
+      </c>
+      <c r="J54" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
+        <v>403</v>
+      </c>
+      <c r="B55" t="s">
+        <v>377</v>
+      </c>
+      <c r="C55">
+        <v>1000</v>
+      </c>
+      <c r="D55">
+        <v>14</v>
+      </c>
+      <c r="E55" t="s">
+        <v>35</v>
+      </c>
+      <c r="F55">
+        <v>0</v>
+      </c>
+      <c r="H55" t="s">
+        <v>58</v>
+      </c>
+      <c r="J55" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
+        <v>403</v>
+      </c>
+      <c r="B56" t="s">
+        <v>377</v>
+      </c>
+      <c r="C56">
+        <v>1000</v>
+      </c>
+      <c r="D56">
+        <v>15</v>
+      </c>
+      <c r="E56" t="s">
+        <v>35</v>
+      </c>
+      <c r="F56">
+        <v>0</v>
+      </c>
+      <c r="H56" t="s">
+        <v>58</v>
+      </c>
+      <c r="J56" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A57" t="s">
+        <v>144</v>
+      </c>
+      <c r="B57" t="s">
+        <v>420</v>
+      </c>
+      <c r="C57">
+        <v>1000</v>
+      </c>
+      <c r="D57">
+        <v>1</v>
+      </c>
+      <c r="E57" t="s">
+        <v>420</v>
+      </c>
+      <c r="F57">
+        <v>0</v>
+      </c>
+      <c r="H57" t="s">
+        <v>58</v>
+      </c>
+      <c r="J57" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
+        <v>144</v>
+      </c>
+      <c r="B58" t="s">
+        <v>420</v>
+      </c>
+      <c r="C58">
+        <v>1000</v>
+      </c>
+      <c r="D58">
+        <v>2</v>
+      </c>
+      <c r="E58" t="s">
+        <v>420</v>
+      </c>
+      <c r="F58">
+        <v>0</v>
+      </c>
+      <c r="H58" t="s">
+        <v>58</v>
+      </c>
+      <c r="J58" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A59" t="s">
+        <v>144</v>
+      </c>
+      <c r="B59" t="s">
+        <v>420</v>
+      </c>
+      <c r="C59">
+        <v>1000</v>
+      </c>
+      <c r="D59">
+        <v>3</v>
+      </c>
+      <c r="E59" t="s">
+        <v>420</v>
+      </c>
+      <c r="F59">
+        <v>0</v>
+      </c>
+      <c r="H59" t="s">
+        <v>58</v>
+      </c>
+      <c r="J59" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A60" t="s">
+        <v>144</v>
+      </c>
+      <c r="B60" t="s">
+        <v>420</v>
+      </c>
+      <c r="C60">
+        <v>1000</v>
+      </c>
+      <c r="D60">
+        <v>4</v>
+      </c>
+      <c r="E60" t="s">
+        <v>420</v>
+      </c>
+      <c r="F60">
+        <v>0</v>
+      </c>
+      <c r="H60" t="s">
+        <v>62</v>
+      </c>
+      <c r="J60" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="61" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A61" t="s">
+        <v>144</v>
+      </c>
+      <c r="B61" t="s">
+        <v>420</v>
+      </c>
+      <c r="C61">
+        <v>1000</v>
+      </c>
+      <c r="D61">
+        <v>5</v>
+      </c>
+      <c r="E61" t="s">
+        <v>420</v>
+      </c>
+      <c r="F61">
+        <v>0</v>
+      </c>
+      <c r="H61" t="s">
+        <v>62</v>
+      </c>
+      <c r="J61" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A62" t="s">
+        <v>145</v>
+      </c>
+      <c r="B62" t="s">
+        <v>420</v>
+      </c>
+      <c r="C62">
+        <v>1000</v>
+      </c>
+      <c r="D62">
+        <v>1</v>
+      </c>
+      <c r="E62" t="s">
+        <v>420</v>
+      </c>
+      <c r="F62">
+        <v>0</v>
+      </c>
+      <c r="H62" t="s">
+        <v>62</v>
+      </c>
+      <c r="J62" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A63" t="s">
+        <v>145</v>
+      </c>
+      <c r="B63" t="s">
+        <v>420</v>
+      </c>
+      <c r="C63">
+        <v>1000</v>
+      </c>
+      <c r="D63">
+        <v>2</v>
+      </c>
+      <c r="E63" t="s">
+        <v>420</v>
+      </c>
+      <c r="F63">
+        <v>0</v>
+      </c>
+      <c r="H63" t="s">
+        <v>62</v>
+      </c>
+      <c r="J63" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A64" t="s">
+        <v>145</v>
+      </c>
+      <c r="B64" t="s">
+        <v>420</v>
+      </c>
+      <c r="C64">
+        <v>1000</v>
+      </c>
+      <c r="D64">
+        <v>3</v>
+      </c>
+      <c r="E64" t="s">
+        <v>420</v>
+      </c>
+      <c r="F64">
+        <v>0</v>
+      </c>
+      <c r="H64" t="s">
+        <v>62</v>
+      </c>
+      <c r="J64" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="65" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A65" t="s">
+        <v>145</v>
+      </c>
+      <c r="B65" t="s">
+        <v>420</v>
+      </c>
+      <c r="C65">
+        <v>1000</v>
+      </c>
+      <c r="D65">
+        <v>4</v>
+      </c>
+      <c r="E65" t="s">
+        <v>420</v>
+      </c>
+      <c r="F65">
+        <v>0</v>
+      </c>
+      <c r="H65" t="s">
+        <v>62</v>
+      </c>
+      <c r="J65" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="66" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A66" t="s">
+        <v>145</v>
+      </c>
+      <c r="B66" t="s">
+        <v>420</v>
+      </c>
+      <c r="C66">
+        <v>1000</v>
+      </c>
+      <c r="D66">
+        <v>5</v>
+      </c>
+      <c r="E66" t="s">
+        <v>420</v>
+      </c>
+      <c r="F66">
+        <v>0</v>
+      </c>
+      <c r="H66" t="s">
+        <v>62</v>
+      </c>
+      <c r="J66" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="67" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A67" t="s">
+        <v>146</v>
+      </c>
+      <c r="B67" t="s">
+        <v>420</v>
+      </c>
+      <c r="C67">
+        <v>1000</v>
+      </c>
+      <c r="D67">
+        <v>1</v>
+      </c>
+      <c r="E67" t="s">
+        <v>420</v>
+      </c>
+      <c r="F67">
+        <v>1</v>
+      </c>
+      <c r="H67" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="68" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A68" t="s">
+        <v>146</v>
+      </c>
+      <c r="B68" t="s">
+        <v>420</v>
+      </c>
+      <c r="C68">
+        <v>1000</v>
+      </c>
+      <c r="D68">
+        <v>2</v>
+      </c>
+      <c r="E68" t="s">
+        <v>420</v>
+      </c>
+      <c r="F68">
+        <v>1</v>
+      </c>
+      <c r="H68" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="69" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A69" t="s">
+        <v>146</v>
+      </c>
+      <c r="B69" t="s">
+        <v>420</v>
+      </c>
+      <c r="C69">
+        <v>1000</v>
+      </c>
+      <c r="D69">
+        <v>3</v>
+      </c>
+      <c r="E69" t="s">
+        <v>420</v>
+      </c>
+      <c r="F69">
+        <v>1</v>
+      </c>
+      <c r="H69" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="70" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A70" t="s">
+        <v>146</v>
+      </c>
+      <c r="B70" t="s">
+        <v>420</v>
+      </c>
+      <c r="C70">
+        <v>1000</v>
+      </c>
+      <c r="D70">
+        <v>4</v>
+      </c>
+      <c r="E70" t="s">
+        <v>420</v>
+      </c>
+      <c r="F70">
+        <v>0</v>
+      </c>
+      <c r="H70" t="s">
+        <v>58</v>
+      </c>
+      <c r="J70" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="71" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A71" t="s">
+        <v>146</v>
+      </c>
+      <c r="B71" t="s">
+        <v>420</v>
+      </c>
+      <c r="C71">
+        <v>1000</v>
+      </c>
+      <c r="D71">
+        <v>5</v>
+      </c>
+      <c r="E71" t="s">
+        <v>420</v>
+      </c>
+      <c r="F71">
+        <v>1</v>
+      </c>
+      <c r="H71" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="72" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A72" t="s">
+        <v>147</v>
+      </c>
+      <c r="B72" t="s">
+        <v>420</v>
+      </c>
+      <c r="C72">
+        <v>1000</v>
+      </c>
+      <c r="D72">
+        <v>1</v>
+      </c>
+      <c r="E72" t="s">
+        <v>420</v>
+      </c>
+      <c r="F72">
+        <v>1</v>
+      </c>
+      <c r="H72" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="73" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A73" t="s">
+        <v>147</v>
+      </c>
+      <c r="B73" t="s">
+        <v>420</v>
+      </c>
+      <c r="C73">
+        <v>1000</v>
+      </c>
+      <c r="D73">
+        <v>2</v>
+      </c>
+      <c r="E73" t="s">
+        <v>420</v>
+      </c>
+      <c r="F73">
+        <v>1</v>
+      </c>
+      <c r="H73" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="74" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A74" t="s">
+        <v>147</v>
+      </c>
+      <c r="B74" t="s">
+        <v>420</v>
+      </c>
+      <c r="C74">
+        <v>1000</v>
+      </c>
+      <c r="D74">
+        <v>3</v>
+      </c>
+      <c r="E74" t="s">
+        <v>420</v>
+      </c>
+      <c r="F74">
+        <v>1</v>
+      </c>
+      <c r="H74" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="75" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A75" t="s">
+        <v>147</v>
+      </c>
+      <c r="B75" t="s">
+        <v>420</v>
+      </c>
+      <c r="C75">
+        <v>1000</v>
+      </c>
+      <c r="D75">
+        <v>4</v>
+      </c>
+      <c r="E75" t="s">
+        <v>420</v>
+      </c>
+      <c r="F75">
+        <v>1</v>
+      </c>
+      <c r="H75" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="76" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A76" t="s">
+        <v>147</v>
+      </c>
+      <c r="B76" t="s">
+        <v>420</v>
+      </c>
+      <c r="C76">
+        <v>1000</v>
+      </c>
+      <c r="D76">
+        <v>5</v>
+      </c>
+      <c r="E76" t="s">
+        <v>420</v>
+      </c>
+      <c r="F76">
+        <v>0</v>
+      </c>
+      <c r="H76" t="s">
+        <v>58</v>
+      </c>
+      <c r="J76" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="77" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A77" t="s">
+        <v>144</v>
+      </c>
+      <c r="B77" t="s">
+        <v>420</v>
+      </c>
+      <c r="C77">
+        <v>2000</v>
+      </c>
+      <c r="D77">
+        <v>1</v>
+      </c>
+      <c r="E77" t="s">
+        <v>420</v>
+      </c>
+      <c r="F77">
+        <v>0</v>
+      </c>
+      <c r="H77" t="s">
+        <v>62</v>
+      </c>
+      <c r="J77" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="78" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A78" t="s">
+        <v>144</v>
+      </c>
+      <c r="B78" t="s">
+        <v>420</v>
+      </c>
+      <c r="C78">
+        <v>2000</v>
+      </c>
+      <c r="D78">
+        <v>2</v>
+      </c>
+      <c r="E78" t="s">
+        <v>420</v>
+      </c>
+      <c r="F78">
+        <v>0</v>
+      </c>
+      <c r="H78" t="s">
+        <v>62</v>
+      </c>
+      <c r="J78" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="79" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A79" t="s">
+        <v>144</v>
+      </c>
+      <c r="B79" t="s">
+        <v>420</v>
+      </c>
+      <c r="C79">
+        <v>2000</v>
+      </c>
+      <c r="D79">
+        <v>3</v>
+      </c>
+      <c r="E79" t="s">
+        <v>420</v>
+      </c>
+      <c r="F79">
+        <v>0</v>
+      </c>
+      <c r="H79" t="s">
+        <v>62</v>
+      </c>
+      <c r="J79" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="80" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A80" t="s">
+        <v>144</v>
+      </c>
+      <c r="B80" t="s">
+        <v>420</v>
+      </c>
+      <c r="C80">
+        <v>2000</v>
+      </c>
+      <c r="D80">
+        <v>4</v>
+      </c>
+      <c r="E80" t="s">
+        <v>420</v>
+      </c>
+      <c r="F80">
+        <v>0</v>
+      </c>
+      <c r="H80" t="s">
+        <v>62</v>
+      </c>
+      <c r="J80" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="81" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A81" t="s">
+        <v>144</v>
+      </c>
+      <c r="B81" t="s">
+        <v>420</v>
+      </c>
+      <c r="C81">
+        <v>2000</v>
+      </c>
+      <c r="D81">
+        <v>5</v>
+      </c>
+      <c r="E81" t="s">
+        <v>420</v>
+      </c>
+      <c r="F81">
+        <v>0</v>
+      </c>
+      <c r="H81" t="s">
+        <v>62</v>
+      </c>
+      <c r="J81" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="82" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A82" t="s">
+        <v>145</v>
+      </c>
+      <c r="B82" t="s">
+        <v>420</v>
+      </c>
+      <c r="C82">
+        <v>2000</v>
+      </c>
+      <c r="D82">
+        <v>1</v>
+      </c>
+      <c r="E82" t="s">
+        <v>420</v>
+      </c>
+      <c r="F82">
+        <v>0</v>
+      </c>
+      <c r="H82" t="s">
+        <v>62</v>
+      </c>
+      <c r="J82" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="83" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A83" t="s">
+        <v>145</v>
+      </c>
+      <c r="B83" t="s">
+        <v>420</v>
+      </c>
+      <c r="C83">
+        <v>2000</v>
+      </c>
+      <c r="D83">
+        <v>2</v>
+      </c>
+      <c r="E83" t="s">
+        <v>420</v>
+      </c>
+      <c r="F83">
+        <v>0</v>
+      </c>
+      <c r="H83" t="s">
+        <v>62</v>
+      </c>
+      <c r="J83" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="84" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A84" t="s">
+        <v>145</v>
+      </c>
+      <c r="B84" t="s">
+        <v>420</v>
+      </c>
+      <c r="C84">
+        <v>2000</v>
+      </c>
+      <c r="D84">
+        <v>3</v>
+      </c>
+      <c r="E84" t="s">
+        <v>420</v>
+      </c>
+      <c r="F84">
+        <v>0</v>
+      </c>
+      <c r="H84" t="s">
+        <v>62</v>
+      </c>
+      <c r="J84" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="85" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A85" t="s">
+        <v>145</v>
+      </c>
+      <c r="B85" t="s">
+        <v>420</v>
+      </c>
+      <c r="C85">
+        <v>2000</v>
+      </c>
+      <c r="D85">
+        <v>4</v>
+      </c>
+      <c r="E85" t="s">
+        <v>420</v>
+      </c>
+      <c r="F85">
+        <v>0</v>
+      </c>
+      <c r="H85" t="s">
+        <v>62</v>
+      </c>
+      <c r="J85" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="86" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A86" t="s">
+        <v>145</v>
+      </c>
+      <c r="B86" t="s">
+        <v>420</v>
+      </c>
+      <c r="C86">
+        <v>2000</v>
+      </c>
+      <c r="D86">
+        <v>5</v>
+      </c>
+      <c r="E86" t="s">
+        <v>420</v>
+      </c>
+      <c r="F86">
+        <v>0</v>
+      </c>
+      <c r="H86" t="s">
+        <v>62</v>
+      </c>
+      <c r="J86" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="87" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A87" t="s">
+        <v>146</v>
+      </c>
+      <c r="B87" t="s">
+        <v>420</v>
+      </c>
+      <c r="C87">
+        <v>2000</v>
+      </c>
+      <c r="D87">
+        <v>1</v>
+      </c>
+      <c r="E87" t="s">
+        <v>420</v>
+      </c>
+      <c r="F87">
+        <v>1</v>
+      </c>
+      <c r="H87" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="88" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A88" t="s">
+        <v>146</v>
+      </c>
+      <c r="B88" t="s">
+        <v>420</v>
+      </c>
+      <c r="C88">
+        <v>2000</v>
+      </c>
+      <c r="D88">
+        <v>2</v>
+      </c>
+      <c r="E88" t="s">
+        <v>420</v>
+      </c>
+      <c r="F88">
+        <v>1</v>
+      </c>
+      <c r="H88" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="89" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A89" t="s">
+        <v>146</v>
+      </c>
+      <c r="B89" t="s">
+        <v>420</v>
+      </c>
+      <c r="C89">
+        <v>2000</v>
+      </c>
+      <c r="D89">
+        <v>3</v>
+      </c>
+      <c r="E89" t="s">
+        <v>420</v>
+      </c>
+      <c r="F89">
+        <v>1</v>
+      </c>
+      <c r="H89" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="90" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A90" t="s">
+        <v>146</v>
+      </c>
+      <c r="B90" t="s">
+        <v>420</v>
+      </c>
+      <c r="C90">
+        <v>2000</v>
+      </c>
+      <c r="D90">
+        <v>4</v>
+      </c>
+      <c r="E90" t="s">
+        <v>420</v>
+      </c>
+      <c r="F90">
+        <v>0</v>
+      </c>
+      <c r="H90" t="s">
+        <v>58</v>
+      </c>
+      <c r="J90" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="91" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A91" t="s">
+        <v>146</v>
+      </c>
+      <c r="B91" t="s">
+        <v>420</v>
+      </c>
+      <c r="C91">
+        <v>2000</v>
+      </c>
+      <c r="D91">
+        <v>5</v>
+      </c>
+      <c r="E91" t="s">
+        <v>420</v>
+      </c>
+      <c r="F91">
+        <v>0</v>
+      </c>
+      <c r="H91" t="s">
+        <v>58</v>
+      </c>
+      <c r="J91" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="92" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A92" t="s">
+        <v>147</v>
+      </c>
+      <c r="B92" t="s">
+        <v>420</v>
+      </c>
+      <c r="C92">
+        <v>2000</v>
+      </c>
+      <c r="D92">
+        <v>1</v>
+      </c>
+      <c r="E92" t="s">
+        <v>420</v>
+      </c>
+      <c r="F92">
+        <v>1</v>
+      </c>
+      <c r="H92" t="s">
+        <v>13</v>
+      </c>
+      <c r="J92" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="93" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A93" t="s">
+        <v>147</v>
+      </c>
+      <c r="B93" t="s">
+        <v>420</v>
+      </c>
+      <c r="C93">
+        <v>2000</v>
+      </c>
+      <c r="D93">
+        <v>2</v>
+      </c>
+      <c r="E93" t="s">
+        <v>420</v>
+      </c>
+      <c r="F93">
+        <v>0</v>
+      </c>
+      <c r="H93" t="s">
+        <v>58</v>
+      </c>
+      <c r="J93" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="94" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A94" t="s">
+        <v>147</v>
+      </c>
+      <c r="B94" t="s">
+        <v>420</v>
+      </c>
+      <c r="C94">
+        <v>2000</v>
+      </c>
+      <c r="D94">
+        <v>3</v>
+      </c>
+      <c r="E94" t="s">
+        <v>420</v>
+      </c>
+      <c r="F94">
+        <v>1</v>
+      </c>
+      <c r="H94" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="95" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A95" t="s">
+        <v>147</v>
+      </c>
+      <c r="B95" t="s">
+        <v>420</v>
+      </c>
+      <c r="C95">
+        <v>2000</v>
+      </c>
+      <c r="D95">
+        <v>4</v>
+      </c>
+      <c r="E95" t="s">
+        <v>420</v>
+      </c>
+      <c r="F95">
+        <v>1</v>
+      </c>
+      <c r="H95" t="s">
+        <v>56</v>
+      </c>
+      <c r="J95" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="96" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A96" t="s">
+        <v>147</v>
+      </c>
+      <c r="B96" t="s">
+        <v>420</v>
+      </c>
+      <c r="C96">
+        <v>2000</v>
+      </c>
+      <c r="D96">
+        <v>5</v>
+      </c>
+      <c r="E96" t="s">
+        <v>420</v>
+      </c>
+      <c r="F96">
+        <v>0</v>
+      </c>
+      <c r="H96" t="s">
+        <v>58</v>
+      </c>
+      <c r="J96" t="s">
+        <v>422</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{76E06697-9F73-9348-BDD7-54FE794126BD}">
+          <x14:formula1>
+            <xm:f>'failure mode options'!$A$2:$A$10</xm:f>
+          </x14:formula1>
+          <xm:sqref>H2:H96</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CBE79B6-38F4-3C44-9FF7-7D936C3A69D9}">
   <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -35952,7 +38589,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3271A2FB-3DCF-6749-BC55-6DF95F82A7E1}">
   <dimension ref="A1:J16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>

</xml_diff>